<commit_message>
Final 50 test cases verification
</commit_message>
<xml_diff>
--- a/IT23622814.xlsx
+++ b/IT23622814.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT23622814\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5062B4EA-2771-4C45-8BBA-5A4BE144C597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_5D85D03E51298B94020683252B36F527575834AB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,6 +40,12 @@
     <t>Status</t>
   </si>
   <si>
+    <t>Singlish input types covered</t>
+  </si>
+  <si>
+    <t>Evidence or Rationale for the input types covered</t>
+  </si>
+  <si>
     <t>Neg_001</t>
   </si>
   <si>
@@ -58,6 +64,12 @@
     <t>FAIL</t>
   </si>
   <si>
+    <t>Question forms</t>
+  </si>
+  <si>
+    <t>Rationale: The overall message is a question as it ends with 'enawada?'.</t>
+  </si>
+  <si>
     <t>Neg_002</t>
   </si>
   <si>
@@ -73,6 +85,9 @@
     <t>බත් කෑවට පස්සේ සෙල්ලම් කරන්න පුළුවන්ද?</t>
   </si>
   <si>
+    <t>Rationale: The overall message is a question as it asks for possibility/permission using 'puluwanda?'.</t>
+  </si>
+  <si>
     <t>Neg_003</t>
   </si>
   <si>
@@ -85,6 +100,12 @@
     <t>ඉක්මනට ඇඳුමක් අඬා ගන්න ගමනක් යන්න, මං එද්දි ලෑස්ති වෙලා ඉන්න.</t>
   </si>
   <si>
+    <t>Command forms</t>
+  </si>
+  <si>
+    <t>Rationale: The input provides a set of directives and instructions ('anda ganna', 'lasthi wela inna').</t>
+  </si>
+  <si>
     <t>Neg_004</t>
   </si>
   <si>
@@ -97,6 +118,9 @@
     <t>රට කෑම ඕනේ නම් පල්ලයහට එන්න</t>
   </si>
   <si>
+    <t>Rationale: Input includes a directive/command to come downstairs using the phrase 'pallayahata enna'.</t>
+  </si>
+  <si>
     <t>Neg_005</t>
   </si>
   <si>
@@ -109,6 +133,9 @@
     <t>Ayubovan! ඔබව සාධාරයෙන් පිළිගනිමු.</t>
   </si>
   <si>
+    <t>Rationale: The input consists of formal salutations and welcoming phrases such as 'Ayubovan!' and 'sadharayen piliganimu'.</t>
+  </si>
+  <si>
     <t>Neg_006</t>
   </si>
   <si>
@@ -121,6 +148,12 @@
     <t>හොදින් විබාගය කරන්න.</t>
   </si>
   <si>
+    <t xml:space="preserve"> Greetings</t>
+  </si>
+  <si>
+    <t>Rationale: The input is a common well-wishing greeting used for exams: 'Hodin vibagaya karanna'.</t>
+  </si>
+  <si>
     <t>Neg_007</t>
   </si>
   <si>
@@ -133,6 +166,12 @@
     <t>අද රට එද්දි මට සරුංගලයක් ගේන්න පුලුවන්ද?.</t>
   </si>
   <si>
+    <t>Requests</t>
+  </si>
+  <si>
+    <t>Rationale: The input is a request for an item using the polite question form 'puluwandha?'.</t>
+  </si>
+  <si>
     <t>Neg_008</t>
   </si>
   <si>
@@ -145,6 +184,9 @@
     <t>මට සපත්තු දෙකක් අරන් දෙන්නකෝ ඉරිදාට කලින්?</t>
   </si>
   <si>
+    <t>Rationale: The input is a request for an action ('aran dennako') within a specific timeframe.</t>
+  </si>
+  <si>
     <t>Neg_009</t>
   </si>
   <si>
@@ -157,6 +199,12 @@
     <t>අනේ හරි නන්දේ මන් ගෙදර ගිහින් බලන්නම්.</t>
   </si>
   <si>
+    <t>Responses</t>
+  </si>
+  <si>
+    <t>Rationale: The input provides a conversational response to a previous statement using 'balannam'.</t>
+  </si>
+  <si>
     <t>Neg_010</t>
   </si>
   <si>
@@ -169,6 +217,9 @@
     <t>හරි මන් වෙලාපහ බස් එකේ ගෙදර එන්නම්.</t>
   </si>
   <si>
+    <t>Rationale: The input acts as a response regarding a future action using the confirmation 'ennam'.</t>
+  </si>
+  <si>
     <t>Neg_011</t>
   </si>
   <si>
@@ -181,6 +232,12 @@
     <t>කතා කර කර ඉන්න එපා.</t>
   </si>
   <si>
+    <t>Repeated Words</t>
+  </si>
+  <si>
+    <t>Rationale: The input includes consecutive repeated words ('katha katha' and 'kara kara') for emphasis.</t>
+  </si>
+  <si>
     <t>Neg_012</t>
   </si>
   <si>
@@ -193,6 +250,9 @@
     <t>දැහෙන්න දෙන්න කතා කරන්න.</t>
   </si>
   <si>
+    <t>Rationale: The input features the repetition of the word 'dhenna' to indicate plurality or intensity.</t>
+  </si>
+  <si>
     <t>Neg_013</t>
   </si>
   <si>
@@ -205,6 +265,12 @@
     <t>අද වැස්ස වහියි?</t>
   </si>
   <si>
+    <t xml:space="preserve"> Inputs with Punctuation Marks</t>
+  </si>
+  <si>
+    <t>Rationale: The input utilizes a question mark (?) to indicate an inquiry about the weather.</t>
+  </si>
+  <si>
     <t>Neg_014</t>
   </si>
   <si>
@@ -217,6 +283,9 @@
     <t>මට උදවු කරන්න; මට අමාරුයි.</t>
   </si>
   <si>
+    <t xml:space="preserve">  Rationale: The input uses a semicolon (;) to separate two independent but related clauses.</t>
+  </si>
+  <si>
     <t>Neg_015</t>
   </si>
   <si>
@@ -229,6 +298,12 @@
     <t>වෙනම් නමක් දාගන්න.</t>
   </si>
   <si>
+    <t xml:space="preserve">     Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Rationale: The word 'dagnn' is a non-standard phonetic spelling variant of 'daganna'.</t>
+  </si>
+  <si>
     <t>Neg_016</t>
   </si>
   <si>
@@ -241,6 +316,12 @@
     <t>ඕන මෘගුලක් කරගන්න.</t>
   </si>
   <si>
+    <t xml:space="preserve">      Romanization / Spelling Variants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Rationale: The word 'mgulak' uses a shortened romanized spelling common in informal chat.</t>
+  </si>
+  <si>
     <t>Neg_017</t>
   </si>
   <si>
@@ -253,6 +334,12 @@
     <t>මගේ mobile phone එක charge කරන්නකෝ.</t>
   </si>
   <si>
+    <t xml:space="preserve">     Isolated English Word Insertions in Singlish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Rationale: Single English words like 'mobile', 'phone', and 'charge' are inserted into the Singlish text.</t>
+  </si>
+  <si>
     <t>Neg_018</t>
   </si>
   <si>
@@ -265,6 +352,12 @@
     <t>ඉරිදාට climate එක ගොඩක් hot.</t>
   </si>
   <si>
+    <t xml:space="preserve">   Isolated English Word Insertions in Singlish</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rationale: Scientific or specific English words like 'climate' and 'hot' are used within the sentence.</t>
+  </si>
+  <si>
     <t>Neg_019</t>
   </si>
   <si>
@@ -277,6 +370,12 @@
     <t>කරුණාකරලා මේක කීප් ඉන් මින්ඩ් තියාගන්න.</t>
   </si>
   <si>
+    <t xml:space="preserve">   Multi-Word English Phrases in Singlish</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rationale: The multi-word English idiomatic phrase 'keep in mind' is inserted inside the Singlish input.</t>
+  </si>
+  <si>
     <t>Neg_020</t>
   </si>
   <si>
@@ -289,6 +388,12 @@
     <t>හැමෝටම උනා keep a distance</t>
   </si>
   <si>
+    <t xml:space="preserve">     Multi-Word English Phrases in Singlish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Rationale: The complete English instructional phrase 'keep  a distance' is used as part of the message.</t>
+  </si>
+  <si>
     <t>Neg_021</t>
   </si>
   <si>
@@ -301,6 +406,12 @@
     <t>කොම්පංච විදියෙ ගත්ත ෆොටෝස් email කරන්න.</t>
   </si>
   <si>
+    <t xml:space="preserve">  English Digital Terms in Singlish</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rationale: The input includes specific digital and technology-related terms such as 'photos' and 'email'.</t>
+  </si>
+  <si>
     <t>Neg_022</t>
   </si>
   <si>
@@ -313,6 +424,12 @@
     <t>ඔයාගේ ගමේ එකේ username එක මොකක්ද?</t>
   </si>
   <si>
+    <t xml:space="preserve"> English Digital Terms in Singlish</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rationale: Input includes digital-specific terminology such as 'username'.</t>
+  </si>
+  <si>
     <t>Neg_023</t>
   </si>
   <si>
@@ -325,6 +442,12 @@
     <t>මම රට project එක GitHub එකට දාන්නම්.</t>
   </si>
   <si>
+    <t xml:space="preserve">   Platform/App Names in Singlish</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rationale: Input includes the name of a specific software development platform: 'GitHub'.</t>
+  </si>
+  <si>
     <t>Neg_024</t>
   </si>
   <si>
@@ -337,6 +460,9 @@
     <t>මම පංචිකාවට්ට ගිහින් Instagram එකට photo එකක් දැම්මා.</t>
   </si>
   <si>
+    <t xml:space="preserve">  Rationale: Input contains a specific social media platform name: 'Instagram'.</t>
+  </si>
+  <si>
     <t>Neg_025</t>
   </si>
   <si>
@@ -349,6 +475,12 @@
     <t>SMS එකක් එවන්න, මම කොමප්ංච විදියෙ ඉන්නෙ.</t>
   </si>
   <si>
+    <t xml:space="preserve">    English Abbreviations/Acronyms in Singlish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Rationale: Input includes the standard telecommunications abbreviation 'SMS'.</t>
+  </si>
+  <si>
     <t>Neg_026</t>
   </si>
   <si>
@@ -361,6 +493,12 @@
     <t>මගේ CV ඒක check කරලා මට චාන්ස් එකක් දෙන්න</t>
   </si>
   <si>
+    <t xml:space="preserve">   English Abbreviations/Acronyms in Singlish</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rationale: Input includes the professional abbreviation 'CV' (Curriculum Vitae).</t>
+  </si>
+  <si>
     <t>Neg_027</t>
   </si>
   <si>
@@ -373,6 +511,12 @@
     <t>මට ඉරිදාට viva එකක් තියෙනවා.</t>
   </si>
   <si>
+    <t xml:space="preserve">  English Clipped Forms in Singlish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Rationale: Input uses the clipped form 'viva' instead of the full term 'viva voce'.</t>
+  </si>
+  <si>
     <t>Neg_028</t>
   </si>
   <si>
@@ -385,6 +529,9 @@
     <t>මට lab එක තියෙන්නේ ඉරිදාට.</t>
   </si>
   <si>
+    <t>Rationale: Input uses the clipped form 'lab' instead of the full term 'laboratory'.</t>
+  </si>
+  <si>
     <t>Neg_029</t>
   </si>
   <si>
@@ -397,6 +544,12 @@
     <t>අපි ඇඳුමක් අඬ ගන්න thailand යමුද?</t>
   </si>
   <si>
+    <t xml:space="preserve">  Place Names Embedded in Singlish</t>
+  </si>
+  <si>
+    <t>Rationale: Input includes the proper noun for a country: 'Thailand'.</t>
+  </si>
+  <si>
     <t>Neg_030</t>
   </si>
   <si>
@@ -409,6 +562,9 @@
     <t>මරිනෝ මල් යන්න අපේ ගෙවල් පැත්තේ එනවාද?</t>
   </si>
   <si>
+    <t>Rationale: Input includes a specific local landmark name: 'Marino Mall'.</t>
+  </si>
+  <si>
     <t>Neg_031</t>
   </si>
   <si>
@@ -421,6 +577,12 @@
     <t>අපි රට දසුන් අයියගේ ගෙදර යනවා.</t>
   </si>
   <si>
+    <t xml:space="preserve">   Person Names Embedded in Singlish</t>
+  </si>
+  <si>
+    <t>Rationale: Input includes the proper name of an individual: 'dasun'.</t>
+  </si>
+  <si>
     <t>Neg_032</t>
   </si>
   <si>
@@ -433,6 +595,12 @@
     <t>උපුල් අයියා මට රට පාටියට එන්න කිව්වා.</t>
   </si>
   <si>
+    <t xml:space="preserve">  Person Names Embedded in Singlish</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rationale: Input includes the proper name of an individual: 'Upul'.</t>
+  </si>
+  <si>
     <t>Neg_033</t>
   </si>
   <si>
@@ -445,6 +613,12 @@
     <t>Science paper එකට ලකුණු 100 ගන්න ප්ලුවන්ධ?</t>
   </si>
   <si>
+    <t xml:space="preserve">   Inputs with Numbers and Numeric Suffixes</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rationale: Input includes a numerical value: '100'.</t>
+  </si>
+  <si>
     <t>Neg_034</t>
   </si>
   <si>
@@ -457,6 +631,9 @@
     <t>මට පරිප්පු ග්රාම් 250 දෙන්නා ප්ලුවන්ධ?</t>
   </si>
   <si>
+    <t xml:space="preserve"> Rationale: Input includes a numerical quantity: '250'.</t>
+  </si>
+  <si>
     <t>Neg_035</t>
   </si>
   <si>
@@ -469,6 +646,12 @@
     <t>නන්දේ, මට Rs.5000 දෙන්නකෝ.</t>
   </si>
   <si>
+    <t xml:space="preserve">   Inputs with Currency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Rationale: Input includes a currency prefix 'Rs.' followed by a numerical value.</t>
+  </si>
+  <si>
     <t>Neg_036</t>
   </si>
   <si>
@@ -481,6 +664,12 @@
     <t>යුරෝ 3000 ගන්න ප්ලුවන්ධ?</t>
   </si>
   <si>
+    <t xml:space="preserve">  Inputs with Currency</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rationale: Input includes a currency name 'Euro' followed by a numerical value.</t>
+  </si>
+  <si>
     <t>Neg_037</t>
   </si>
   <si>
@@ -493,6 +682,12 @@
     <t>ඔයා 04.00 PM වෙද්දි එන්න ප්ලුවන්ධ?</t>
   </si>
   <si>
+    <t xml:space="preserve">   Inputs with Time Formats</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rationale: The input includes a specific clock time using the 12-hour format '04.00 PM'.</t>
+  </si>
+  <si>
     <t>Neg_038</t>
   </si>
   <si>
@@ -505,6 +700,12 @@
     <t>ඔයා 04.00 PM වෙද්දි මට්ටකුලිය යනවා.</t>
   </si>
   <si>
+    <t xml:space="preserve">    Inputs with Time Formats</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rationale: The input combines a time format ('04.00 PM') with a local place name ('mattakuliya').</t>
+  </si>
+  <si>
     <t>Neg_039</t>
   </si>
   <si>
@@ -517,6 +718,12 @@
     <t>මාර්තු 15 ට කලින් form එක ගමට ඇවිත් දෙන්න.</t>
   </si>
   <si>
+    <t xml:space="preserve">   Inputs with Dates</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rationale: The input contains a specific calendar date 'march 15' within the Singlish text.</t>
+  </si>
+  <si>
     <t>Neg_040</t>
   </si>
   <si>
@@ -529,6 +736,12 @@
     <t>ඊළඟ meeting එක 2026-06-05 ඉරිදාට තියනවා.</t>
   </si>
   <si>
+    <t xml:space="preserve">    Inputs with Dates</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rationale: Input includes a numerical date in the YYYY-MM-DD format: '2026-06-05'. </t>
+  </si>
+  <si>
     <t>Neg_041</t>
   </si>
   <si>
@@ -541,6 +754,12 @@
     <t>මේ බිත්තරේ බර ග්රාම් 30</t>
   </si>
   <si>
+    <t xml:space="preserve">   Inputs with Unit of Measurements</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rationale: Input includes a numerical weight value with its unit: 'gram 30'.</t>
+  </si>
+  <si>
     <t>Neg_042</t>
   </si>
   <si>
@@ -553,6 +772,12 @@
     <t>මගේ අගේ බර කිලෝගල් 20</t>
   </si>
   <si>
+    <t xml:space="preserve">    Inputs with Unit of Measurements</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rationale: Input includes a complex unit of measurement: 'kilogram 20'.</t>
+  </si>
+  <si>
     <t>Neg_043</t>
   </si>
   <si>
@@ -565,6 +790,12 @@
     <t>රා වෙන්න කලින් ගෙදර වරෙන්</t>
   </si>
   <si>
+    <t xml:space="preserve">   Inputs with Slang and Casual Phrasing</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rationale: Input includes highly informal, casual directives such as 'waren'.</t>
+  </si>
+  <si>
     <t>Neg_044</t>
   </si>
   <si>
@@ -577,6 +808,9 @@
     <t>රට රවුම් ගහන්න එපා යකෝ</t>
   </si>
   <si>
+    <t xml:space="preserve"> Rationale: Input contains informal colloquial terms like 'yako' used for emphasis.</t>
+  </si>
+  <si>
     <t>Neg_045</t>
   </si>
   <si>
@@ -589,6 +823,12 @@
     <t>අලුත් update එක www.ගූගල්.කොම් එකෙන් බලන්න.</t>
   </si>
   <si>
+    <t xml:space="preserve">    Online Indentifiers in Singlish</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Rationale: Input contains a web URL identifier: 'www.google.com'.</t>
+  </si>
+  <si>
     <t>Neg_046</t>
   </si>
   <si>
@@ -601,6 +841,9 @@
     <t>මේ browser එකෙන් යන්න www.යහෝ.කොම්</t>
   </si>
   <si>
+    <t>Rationale: Input contains a web URL identifier: 'www.google.com'.</t>
+  </si>
+  <si>
     <t>Neg_047</t>
   </si>
   <si>
@@ -613,6 +856,12 @@
     <t>සුබ උපන් දිනයක් වේවා!</t>
   </si>
   <si>
+    <t xml:space="preserve">  Inputs Containing Emojis</t>
+  </si>
+  <si>
+    <t>Rationale: Input includes a celebration emoji character: '🎂'.</t>
+  </si>
+  <si>
     <t>Neg_048</t>
   </si>
   <si>
@@ -625,6 +874,9 @@
     <t>අපි මේක ඉවර කරමු 🤣</t>
   </si>
   <si>
+    <t>Rationale: Input includes a graphical bicep emoji representing effort: '💪'.</t>
+  </si>
+  <si>
     <t>Neg_049</t>
   </si>
   <si>
@@ -637,6 +889,9 @@
     <t>ඔයා හෙට එනවද? 😅</t>
   </si>
   <si>
+    <t>Rationale: Input includes a thinking face emoji character: '🤔'.</t>
+  </si>
+  <si>
     <t>Neg_050</t>
   </si>
   <si>
@@ -649,265 +904,10 @@
     <t>news බලන්න මේ link එකෙන් යන්න www.news.ල්ක්</t>
   </si>
   <si>
-    <t>Singlish input types covered</t>
-  </si>
-  <si>
-    <t>Evidence or Rationale for the input types covered</t>
-  </si>
-  <si>
-    <t>Question forms</t>
-  </si>
-  <si>
-    <t>Command forms</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Greetings</t>
-  </si>
-  <si>
-    <t>Requests</t>
-  </si>
-  <si>
-    <t>Responses</t>
-  </si>
-  <si>
-    <t>Repeated Words</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Inputs with Punctuation Marks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">     Romanization / Spelling Variants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      Romanization / Spelling Variants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">     Isolated English Word Insertions in Singlish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Isolated English Word Insertions in Singlish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Multi-Word English Phrases in Singlish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">     Multi-Word English Phrases in Singlish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  English Digital Terms in Singlish</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> English Digital Terms in Singlish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Platform/App Names in Singlish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    English Abbreviations/Acronyms in Singlish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   English Abbreviations/Acronyms in Singlish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  English Clipped Forms in Singlish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Place Names Embedded in Singlish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Person Names Embedded in Singlish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Person Names Embedded in Singlish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Inputs with Numbers and Numeric Suffixes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Inputs with Currency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Inputs with Currency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Inputs with Time Formats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Inputs with Time Formats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Inputs with Dates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Inputs with Dates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Inputs with Unit of Measurements</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Inputs with Unit of Measurements</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Inputs with Slang and Casual Phrasing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Online Indentifiers in Singlish</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Inputs Containing Emojis</t>
-  </si>
-  <si>
     <t xml:space="preserve">  Online Indentifiers in Singlish</t>
   </si>
   <si>
-    <t>Rationale: The overall message is a question as it ends with 'enawada?'.</t>
-  </si>
-  <si>
-    <t>Rationale: The overall message is a question as it asks for possibility/permission using 'puluwanda?'.</t>
-  </si>
-  <si>
-    <t>Rationale: The input provides a set of directives and instructions ('anda ganna', 'lasthi wela inna').</t>
-  </si>
-  <si>
-    <t>Rationale: Input includes a directive/command to come downstairs using the phrase 'pallayahata enna'.</t>
-  </si>
-  <si>
-    <t>Rationale: The input consists of formal salutations and welcoming phrases such as 'Ayubovan!' and 'sadharayen piliganimu'.</t>
-  </si>
-  <si>
-    <t>Rationale: The input is a common well-wishing greeting used for exams: 'Hodin vibagaya karanna'.</t>
-  </si>
-  <si>
-    <t>Rationale: The input is a request for an item using the polite question form 'puluwandha?'.</t>
-  </si>
-  <si>
-    <t>Rationale: The input is a request for an action ('aran dennako') within a specific timeframe.</t>
-  </si>
-  <si>
-    <t>Rationale: The input provides a conversational response to a previous statement using 'balannam'.</t>
-  </si>
-  <si>
-    <t>Rationale: The input acts as a response regarding a future action using the confirmation 'ennam'.</t>
-  </si>
-  <si>
-    <t>Rationale: The input includes consecutive repeated words ('katha katha' and 'kara kara') for emphasis.</t>
-  </si>
-  <si>
-    <t>Rationale: The input features the repetition of the word 'dhenna' to indicate plurality or intensity.</t>
-  </si>
-  <si>
-    <t>Rationale: The input utilizes a question mark (?) to indicate an inquiry about the weather.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Rationale: The input uses a semicolon (;) to separate two independent but related clauses.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Rationale: The word 'dagnn' is a non-standard phonetic spelling variant of 'daganna'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Rationale: The word 'mgulak' uses a shortened romanized spelling common in informal chat.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Rationale: Single English words like 'mobile', 'phone', and 'charge' are inserted into the Singlish text.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: Scientific or specific English words like 'climate' and 'hot' are used within the sentence.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: The multi-word English idiomatic phrase 'keep in mind' is inserted inside the Singlish input.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Rationale: The complete English instructional phrase 'keep  a distance' is used as part of the message.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: The input includes specific digital and technology-related terms such as 'photos' and 'email'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: Input includes digital-specific terminology such as 'username'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: Input includes the name of a specific software development platform: 'GitHub'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Rationale: Input contains a specific social media platform name: 'Instagram'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Rationale: Input includes the standard telecommunications abbreviation 'SMS'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: Input includes the professional abbreviation 'CV' (Curriculum Vitae).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Rationale: Input uses the clipped form 'viva' instead of the full term 'viva voce'.</t>
-  </si>
-  <si>
-    <t>Rationale: Input uses the clipped form 'lab' instead of the full term 'laboratory'.</t>
-  </si>
-  <si>
-    <t>Rationale: Input includes the proper noun for a country: 'Thailand'.</t>
-  </si>
-  <si>
-    <t>Rationale: Input includes a specific local landmark name: 'Marino Mall'.</t>
-  </si>
-  <si>
-    <t>Rationale: Input includes the proper name of an individual: 'dasun'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: Input includes the proper name of an individual: 'Upul'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: Input includes a numerical value: '100'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: Input includes a numerical quantity: '250'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Rationale: Input includes a currency prefix 'Rs.' followed by a numerical value.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: Input includes a currency name 'Euro' followed by a numerical value.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: The input includes a specific clock time using the 12-hour format '04.00 PM'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: The input combines a time format ('04.00 PM') with a local place name ('mattakuliya').</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: The input contains a specific calendar date 'march 15' within the Singlish text.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: Input includes a numerical date in the YYYY-MM-DD format: '2026-06-05'. </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: Input includes a numerical weight value with its unit: 'gram 30'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: Input includes a complex unit of measurement: 'kilogram 20'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: Input includes highly informal, casual directives such as 'waren'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: Input contains informal colloquial terms like 'yako' used for emphasis.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Rationale: Input contains a web URL identifier: 'www.google.com'.</t>
-  </si>
-  <si>
-    <t>Rationale: Input includes a celebration emoji character: '🎂'.</t>
-  </si>
-  <si>
-    <t>Rationale: Input includes a graphical bicep emoji representing effort: '💪'.</t>
-  </si>
-  <si>
-    <t>Rationale: Input includes a thinking face emoji character: '🤔'.</t>
-  </si>
-  <si>
     <t>Rationale: Input includes a specific website link identifier: 'www.news.lk'.</t>
-  </si>
-  <si>
-    <t>Rationale: Input contains a web URL identifier: 'www.google.com'.</t>
   </si>
 </sst>
 </file>
@@ -1013,12 +1013,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
@@ -1341,36 +1341,36 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>209</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>210</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="2" t="s">
         <v>8</v>
       </c>
+      <c r="B2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>10</v>
+      </c>
       <c r="D2" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>246</v>
+        <v>12</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1405,28 +1405,28 @@
     </row>
     <row r="6" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>247</v>
+      <c r="H6" s="2" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1461,28 +1461,28 @@
     </row>
     <row r="10" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>18</v>
+      <c r="C10" s="5" t="s">
+        <v>23</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>248</v>
+        <v>25</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1517,28 +1517,28 @@
     </row>
     <row r="14" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>22</v>
+        <v>28</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>29</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>249</v>
+        <v>31</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1573,26 +1573,26 @@
     </row>
     <row r="18" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>26</v>
+        <v>33</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>34</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5" t="s">
-        <v>250</v>
+        <v>36</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1627,28 +1627,28 @@
     </row>
     <row r="22" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>30</v>
+        <v>38</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>39</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G22" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="H22" s="5" t="s">
-        <v>251</v>
+        <v>41</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1683,28 +1683,28 @@
     </row>
     <row r="26" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>34</v>
+        <v>44</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>45</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="H26" s="5" t="s">
-        <v>252</v>
+        <v>47</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1739,28 +1739,28 @@
     </row>
     <row r="30" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>38</v>
+        <v>50</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="F30" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="H30" s="5" t="s">
-        <v>253</v>
+        <v>53</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1795,28 +1795,28 @@
     </row>
     <row r="34" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>42</v>
+        <v>55</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>56</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="F34" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G34" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="H34" s="5" t="s">
-        <v>254</v>
+        <v>58</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1851,28 +1851,28 @@
     </row>
     <row r="38" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>46</v>
+        <v>61</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>62</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="F38" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G38" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="H38" s="5" t="s">
-        <v>255</v>
+        <v>64</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1907,28 +1907,28 @@
     </row>
     <row r="42" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>50</v>
+        <v>66</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>67</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>51</v>
+        <v>68</v>
       </c>
       <c r="E42" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="F42" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G42" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="H42" s="5" t="s">
-        <v>256</v>
+        <v>69</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1963,28 +1963,28 @@
     </row>
     <row r="46" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B46" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>54</v>
+        <v>72</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>73</v>
       </c>
       <c r="D46" s="7" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="E46" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="F46" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G46" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="H46" s="5" t="s">
-        <v>257</v>
+        <v>75</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2019,28 +2019,28 @@
     </row>
     <row r="50" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B50" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>58</v>
+        <v>77</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>78</v>
       </c>
       <c r="D50" s="7" t="s">
-        <v>59</v>
+        <v>79</v>
       </c>
       <c r="E50" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="F50" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G50" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="H50" s="5" t="s">
-        <v>258</v>
+        <v>80</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2075,28 +2075,28 @@
     </row>
     <row r="54" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="B54" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="F54" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G54" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="H54" s="2" t="s">
-        <v>259</v>
+        <v>83</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="E54" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="F54" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G54" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="H54" s="5" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="55" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2131,28 +2131,28 @@
     </row>
     <row r="58" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="B58" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="F58" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G58" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="H58" s="2" t="s">
-        <v>260</v>
+        <v>88</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="E58" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="F58" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G58" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="H58" s="5" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="59" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2187,28 +2187,28 @@
     </row>
     <row r="62" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="B62" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="E62" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="F62" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G62" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="H62" s="2" t="s">
-        <v>261</v>
+        <v>94</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C62" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="D62" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="E62" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="F62" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G62" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="H62" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="63" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2243,28 +2243,28 @@
     </row>
     <row r="66" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="B66" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="F66" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G66" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="H66" s="2" t="s">
-        <v>262</v>
+        <v>100</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C66" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D66" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="E66" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="F66" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G66" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="H66" s="5" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="67" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2299,28 +2299,28 @@
     </row>
     <row r="70" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="B70" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C70" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="E70" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="F70" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G70" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="H70" s="2" t="s">
-        <v>263</v>
+        <v>106</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C70" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="D70" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="F70" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G70" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="H70" s="5" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="71" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2355,28 +2355,28 @@
     </row>
     <row r="74" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="B74" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D74" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="E74" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F74" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G74" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="H74" s="2" t="s">
-        <v>264</v>
+        <v>112</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C74" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="D74" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="E74" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="F74" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G74" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="H74" s="5" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2411,28 +2411,28 @@
     </row>
     <row r="78" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="B78" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="E78" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F78" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G78" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="H78" s="2" t="s">
-        <v>265</v>
+        <v>118</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C78" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="D78" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="E78" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="F78" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G78" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="H78" s="5" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="79" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2467,28 +2467,28 @@
     </row>
     <row r="82" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="B82" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="E82" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F82" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G82" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="H82" s="2" t="s">
-        <v>266</v>
+        <v>124</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C82" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D82" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="E82" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="F82" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G82" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="H82" s="5" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="83" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2523,28 +2523,28 @@
     </row>
     <row r="86" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="B86" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="D86" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="E86" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="F86" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G86" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="H86" s="2" t="s">
-        <v>267</v>
+        <v>130</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C86" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D86" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="E86" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="F86" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G86" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="H86" s="5" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="87" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2579,28 +2579,28 @@
     </row>
     <row r="90" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="B90" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="D90" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="E90" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="F90" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G90" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="H90" s="2" t="s">
-        <v>268</v>
+        <v>136</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C90" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="D90" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="E90" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="F90" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G90" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="H90" s="5" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="91" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2635,28 +2635,28 @@
     </row>
     <row r="94" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="B94" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C94" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="D94" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="E94" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="F94" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G94" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="H94" s="2" t="s">
-        <v>269</v>
+        <v>142</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C94" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="D94" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="E94" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="F94" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G94" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="H94" s="5" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="95" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2691,28 +2691,28 @@
     </row>
     <row r="98" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="B98" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C98" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D98" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="E98" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F98" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G98" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="H98" s="2" t="s">
-        <v>270</v>
+        <v>147</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C98" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="D98" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="E98" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="F98" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G98" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="H98" s="5" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="99" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2747,28 +2747,28 @@
     </row>
     <row r="102" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="B102" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C102" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D102" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="E102" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="F102" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G102" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="H102" s="2" t="s">
-        <v>271</v>
+        <v>153</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C102" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="D102" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="E102" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="F102" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G102" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="H102" s="5" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="103" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2803,28 +2803,28 @@
     </row>
     <row r="106" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="B106" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C106" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="D106" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="E106" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="F106" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G106" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="H106" s="2" t="s">
-        <v>272</v>
+        <v>159</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C106" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D106" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="E106" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="F106" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G106" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="H106" s="5" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="107" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2859,28 +2859,28 @@
     </row>
     <row r="110" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="B110" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C110" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="D110" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="E110" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="F110" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G110" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="H110" s="2" t="s">
-        <v>273</v>
+        <v>165</v>
+      </c>
+      <c r="B110" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C110" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="D110" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="E110" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="F110" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G110" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="H110" s="5" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="111" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2915,28 +2915,28 @@
     </row>
     <row r="114" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="B114" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C114" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="D114" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="E114" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="F114" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G114" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="H114" s="2" t="s">
-        <v>274</v>
+        <v>170</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C114" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="D114" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="E114" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="F114" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G114" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="H114" s="5" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="115" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -2971,28 +2971,28 @@
     </row>
     <row r="118" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="B118" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C118" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="D118" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="E118" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="F118" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G118" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="H118" s="2" t="s">
-        <v>275</v>
+        <v>176</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C118" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="D118" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="E118" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="F118" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G118" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="H118" s="5" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="119" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3027,28 +3027,28 @@
     </row>
     <row r="122" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="B122" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C122" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="D122" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="E122" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="F122" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G122" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="H122" s="2" t="s">
-        <v>276</v>
+        <v>181</v>
+      </c>
+      <c r="B122" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C122" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="D122" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="E122" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="F122" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G122" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="H122" s="5" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="123" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3083,28 +3083,28 @@
     </row>
     <row r="126" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="B126" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C126" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="D126" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="E126" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="F126" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G126" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="H126" s="2" t="s">
-        <v>277</v>
+        <v>187</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C126" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="D126" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="E126" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="F126" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G126" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="H126" s="5" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="127" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3139,28 +3139,28 @@
     </row>
     <row r="130" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="B130" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C130" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="D130" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="E130" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="F130" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G130" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="H130" s="2" t="s">
-        <v>278</v>
+        <v>193</v>
+      </c>
+      <c r="B130" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C130" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="D130" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="E130" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="F130" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G130" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="H130" s="5" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="131" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3195,28 +3195,28 @@
     </row>
     <row r="134" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="B134" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C134" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="D134" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="E134" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="F134" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G134" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="H134" s="2" t="s">
-        <v>279</v>
+        <v>199</v>
+      </c>
+      <c r="B134" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C134" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="D134" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="E134" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="F134" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G134" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="H134" s="5" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="135" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3251,28 +3251,28 @@
     </row>
     <row r="138" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="B138" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C138" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="D138" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="E138" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="F138" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G138" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="H138" s="2" t="s">
-        <v>280</v>
+        <v>204</v>
+      </c>
+      <c r="B138" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C138" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="D138" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="E138" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="F138" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G138" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="H138" s="5" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="139" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3307,28 +3307,28 @@
     </row>
     <row r="142" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="B142" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C142" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="D142" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="E142" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F142" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G142" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="H142" s="2" t="s">
-        <v>281</v>
+        <v>210</v>
+      </c>
+      <c r="B142" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C142" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="D142" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="E142" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="F142" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G142" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="H142" s="5" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="143" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3363,28 +3363,28 @@
     </row>
     <row r="146" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="B146" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C146" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="D146" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="E146" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="F146" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G146" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="H146" s="2" t="s">
-        <v>282</v>
+        <v>216</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C146" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="D146" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="E146" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="F146" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G146" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="H146" s="5" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="147" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3419,28 +3419,28 @@
     </row>
     <row r="150" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="B150" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C150" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="D150" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="E150" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="F150" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G150" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="H150" s="2" t="s">
-        <v>283</v>
+        <v>222</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C150" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D150" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="E150" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="F150" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G150" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="H150" s="5" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="151" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3475,28 +3475,28 @@
     </row>
     <row r="154" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A154" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="B154" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C154" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="D154" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="E154" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="F154" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G154" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="H154" s="2" t="s">
-        <v>284</v>
+        <v>228</v>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C154" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="D154" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="E154" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="F154" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G154" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="H154" s="5" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="155" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3531,28 +3531,28 @@
     </row>
     <row r="158" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="B158" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C158" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="D158" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="E158" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="F158" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G158" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B158" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C158" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="D158" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="E158" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="F158" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G158" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="H158" s="5" t="s">
         <v>239</v>
-      </c>
-      <c r="H158" s="2" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="159" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3587,28 +3587,28 @@
     </row>
     <row r="162" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A162" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="B162" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C162" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="D162" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="E162" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="F162" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G162" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="H162" s="2" t="s">
-        <v>286</v>
+      <c r="B162" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C162" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="D162" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="E162" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="F162" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G162" s="5" t="s">
+        <v>244</v>
+      </c>
+      <c r="H162" s="5" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="163" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3643,28 +3643,28 @@
     </row>
     <row r="166" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A166" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="B166" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C166" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="D166" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="E166" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="F166" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G166" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="H166" s="2" t="s">
-        <v>287</v>
+        <v>246</v>
+      </c>
+      <c r="B166" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C166" s="5" t="s">
+        <v>247</v>
+      </c>
+      <c r="D166" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="E166" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="F166" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G166" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="H166" s="5" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="167" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3699,28 +3699,28 @@
     </row>
     <row r="170" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A170" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="B170" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C170" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="D170" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="E170" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="F170" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G170" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="H170" s="2" t="s">
-        <v>288</v>
+        <v>252</v>
+      </c>
+      <c r="B170" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C170" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="D170" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="E170" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="F170" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G170" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="H170" s="5" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="171" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3755,28 +3755,28 @@
     </row>
     <row r="174" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A174" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="B174" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C174" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="D174" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="E174" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="F174" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G174" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="H174" s="2" t="s">
-        <v>289</v>
+        <v>258</v>
+      </c>
+      <c r="B174" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C174" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="D174" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="E174" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="F174" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G174" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="H174" s="5" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="175" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3811,28 +3811,28 @@
     </row>
     <row r="178" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A178" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="B178" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C178" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="D178" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="E178" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="F178" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G178" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="H178" s="2" t="s">
-        <v>290</v>
+        <v>263</v>
+      </c>
+      <c r="B178" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C178" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="D178" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="E178" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="F178" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G178" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="H178" s="5" t="s">
+        <v>268</v>
       </c>
     </row>
     <row r="179" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3867,28 +3867,28 @@
     </row>
     <row r="182" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A182" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="B182" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C182" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="D182" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E182" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="F182" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G182" s="2" t="s">
-        <v>243</v>
-      </c>
-      <c r="H182" s="2" t="s">
-        <v>295</v>
+        <v>269</v>
+      </c>
+      <c r="B182" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C182" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="D182" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="E182" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="F182" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G182" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="H182" s="5" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="183" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3923,28 +3923,28 @@
     </row>
     <row r="186" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A186" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="B186" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C186" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="D186" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="E186" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="F186" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G186" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="H186" s="2" t="s">
-        <v>291</v>
+        <v>274</v>
+      </c>
+      <c r="B186" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C186" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="D186" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="E186" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="F186" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G186" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="H186" s="5" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="187" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3979,28 +3979,28 @@
     </row>
     <row r="190" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A190" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="B190" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C190" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="D190" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="E190" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="F190" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G190" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="H190" s="2" t="s">
-        <v>292</v>
+        <v>280</v>
+      </c>
+      <c r="B190" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C190" s="5" t="s">
+        <v>281</v>
+      </c>
+      <c r="D190" s="5" t="s">
+        <v>282</v>
+      </c>
+      <c r="E190" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="F190" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G190" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="H190" s="5" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="191" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4035,28 +4035,28 @@
     </row>
     <row r="194" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A194" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="B194" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C194" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="D194" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="E194" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="F194" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G194" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="H194" s="2" t="s">
-        <v>293</v>
+        <v>285</v>
+      </c>
+      <c r="B194" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C194" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="D194" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="E194" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="F194" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G194" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="H194" s="5" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="195" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4091,28 +4091,28 @@
     </row>
     <row r="198" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A198" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="B198" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C198" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="D198" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="E198" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="F198" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G198" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="H198" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B198" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C198" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="D198" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="E198" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="F198" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G198" s="5" t="s">
         <v>294</v>
+      </c>
+      <c r="H198" s="5" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="199" spans="1:8" ht="49.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4147,232 +4147,338 @@
     </row>
   </sheetData>
   <mergeCells count="400">
+    <mergeCell ref="C6:C9"/>
+    <mergeCell ref="C62:C65"/>
+    <mergeCell ref="E62:E65"/>
+    <mergeCell ref="H6:H9"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="H98:H101"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="B98:B101"/>
+    <mergeCell ref="D154:D157"/>
+    <mergeCell ref="F154:F157"/>
+    <mergeCell ref="A158:A161"/>
+    <mergeCell ref="G174:G177"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="E46:E49"/>
+    <mergeCell ref="D106:D109"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="E86:E89"/>
+    <mergeCell ref="B162:B165"/>
+    <mergeCell ref="G150:G153"/>
+    <mergeCell ref="G94:G97"/>
+    <mergeCell ref="H126:H129"/>
+    <mergeCell ref="G158:G161"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="D22:D25"/>
+    <mergeCell ref="F78:F81"/>
+    <mergeCell ref="H78:H81"/>
+    <mergeCell ref="B86:B89"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="G58:G61"/>
+    <mergeCell ref="A150:A153"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="H186:H189"/>
+    <mergeCell ref="D26:D29"/>
+    <mergeCell ref="D82:D85"/>
+    <mergeCell ref="F82:F85"/>
+    <mergeCell ref="H30:H33"/>
+    <mergeCell ref="B90:B93"/>
+    <mergeCell ref="A94:A97"/>
+    <mergeCell ref="F146:F149"/>
+    <mergeCell ref="H146:H149"/>
+    <mergeCell ref="G126:G129"/>
+    <mergeCell ref="H10:H13"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="H58:H61"/>
+    <mergeCell ref="C22:C25"/>
+    <mergeCell ref="E122:E125"/>
+    <mergeCell ref="E78:E81"/>
+    <mergeCell ref="G122:G125"/>
+    <mergeCell ref="G78:G81"/>
+    <mergeCell ref="C134:C137"/>
+    <mergeCell ref="E186:E189"/>
+    <mergeCell ref="D198:D201"/>
+    <mergeCell ref="F198:F201"/>
+    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="E90:E93"/>
+    <mergeCell ref="F110:F113"/>
+    <mergeCell ref="H110:H113"/>
+    <mergeCell ref="B166:B169"/>
+    <mergeCell ref="E154:E157"/>
+    <mergeCell ref="B158:B161"/>
+    <mergeCell ref="G154:G157"/>
+    <mergeCell ref="H174:H177"/>
+    <mergeCell ref="G186:G189"/>
+    <mergeCell ref="G142:G145"/>
+    <mergeCell ref="C138:C141"/>
+    <mergeCell ref="B174:B177"/>
+    <mergeCell ref="A82:A85"/>
+    <mergeCell ref="E106:E109"/>
+    <mergeCell ref="H134:H137"/>
+    <mergeCell ref="G106:G109"/>
+    <mergeCell ref="E198:E201"/>
+    <mergeCell ref="G198:G201"/>
+    <mergeCell ref="G170:G173"/>
+    <mergeCell ref="D90:D93"/>
+    <mergeCell ref="E194:E197"/>
+    <mergeCell ref="A190:A193"/>
+    <mergeCell ref="C190:C193"/>
+    <mergeCell ref="D74:D77"/>
+    <mergeCell ref="B138:B141"/>
+    <mergeCell ref="D138:D141"/>
+    <mergeCell ref="A142:A145"/>
     <mergeCell ref="C14:C17"/>
-    <mergeCell ref="B66:B69"/>
-    <mergeCell ref="C154:C157"/>
-    <mergeCell ref="C98:C101"/>
     <mergeCell ref="E14:E17"/>
+    <mergeCell ref="G70:G73"/>
+    <mergeCell ref="E30:E33"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="C46:C49"/>
+    <mergeCell ref="D14:D17"/>
+    <mergeCell ref="F14:F17"/>
+    <mergeCell ref="D86:D89"/>
+    <mergeCell ref="F86:F89"/>
+    <mergeCell ref="F142:F145"/>
+    <mergeCell ref="G18:G21"/>
+    <mergeCell ref="E34:E37"/>
+    <mergeCell ref="B182:B185"/>
+    <mergeCell ref="G34:G37"/>
+    <mergeCell ref="D162:D165"/>
+    <mergeCell ref="C130:C133"/>
+    <mergeCell ref="G30:G33"/>
+    <mergeCell ref="C194:C197"/>
+    <mergeCell ref="G110:G113"/>
+    <mergeCell ref="H150:H153"/>
+    <mergeCell ref="C18:C21"/>
+    <mergeCell ref="E18:E21"/>
+    <mergeCell ref="B150:B153"/>
+    <mergeCell ref="B190:B193"/>
+    <mergeCell ref="C26:C29"/>
+    <mergeCell ref="D190:D193"/>
+    <mergeCell ref="E82:E85"/>
+    <mergeCell ref="G82:G85"/>
+    <mergeCell ref="H102:H105"/>
+    <mergeCell ref="G146:G149"/>
+    <mergeCell ref="D122:D125"/>
+    <mergeCell ref="C90:C93"/>
+    <mergeCell ref="F122:F125"/>
+    <mergeCell ref="C182:C185"/>
+    <mergeCell ref="H178:H181"/>
+    <mergeCell ref="E182:E185"/>
+    <mergeCell ref="F186:F189"/>
+    <mergeCell ref="H42:H45"/>
+    <mergeCell ref="G194:G197"/>
+    <mergeCell ref="H50:H53"/>
+    <mergeCell ref="H142:H145"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="C2:C5"/>
+    <mergeCell ref="E2:E5"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="D98:D101"/>
+    <mergeCell ref="C66:C69"/>
+    <mergeCell ref="H62:H65"/>
+    <mergeCell ref="F98:F101"/>
+    <mergeCell ref="A102:A105"/>
+    <mergeCell ref="E66:E69"/>
+    <mergeCell ref="C102:C105"/>
+    <mergeCell ref="D50:D53"/>
+    <mergeCell ref="G86:G89"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="D2:D5"/>
+    <mergeCell ref="F18:F21"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="F22:F25"/>
+    <mergeCell ref="H22:H25"/>
+    <mergeCell ref="E54:E57"/>
+    <mergeCell ref="G54:G57"/>
+    <mergeCell ref="H86:H89"/>
+    <mergeCell ref="D38:D41"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="D6:D9"/>
+    <mergeCell ref="G178:G181"/>
+    <mergeCell ref="F6:F9"/>
+    <mergeCell ref="B62:B65"/>
+    <mergeCell ref="E98:E101"/>
+    <mergeCell ref="G162:G165"/>
+    <mergeCell ref="C150:C153"/>
+    <mergeCell ref="E22:E25"/>
+    <mergeCell ref="G22:G25"/>
+    <mergeCell ref="E134:E137"/>
+    <mergeCell ref="F54:F57"/>
+    <mergeCell ref="C158:C161"/>
+    <mergeCell ref="B50:B53"/>
+    <mergeCell ref="E38:E41"/>
+    <mergeCell ref="G38:G41"/>
+    <mergeCell ref="G98:G101"/>
+    <mergeCell ref="D174:D177"/>
+    <mergeCell ref="F174:F177"/>
+    <mergeCell ref="D166:D169"/>
+    <mergeCell ref="B118:B121"/>
+    <mergeCell ref="E130:E133"/>
+    <mergeCell ref="B134:B137"/>
+    <mergeCell ref="G130:G133"/>
+    <mergeCell ref="G114:G117"/>
+    <mergeCell ref="H198:H201"/>
+    <mergeCell ref="D42:D45"/>
+    <mergeCell ref="G90:G93"/>
+    <mergeCell ref="D94:D97"/>
+    <mergeCell ref="A114:A117"/>
+    <mergeCell ref="A170:A173"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="C170:C173"/>
+    <mergeCell ref="F158:F161"/>
+    <mergeCell ref="H54:H57"/>
     <mergeCell ref="A166:A169"/>
-    <mergeCell ref="E102:E105"/>
-    <mergeCell ref="B50:B53"/>
-    <mergeCell ref="A162:A165"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="D26:D29"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="C18:C21"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="E18:E21"/>
-    <mergeCell ref="D22:D25"/>
-    <mergeCell ref="F30:F33"/>
+    <mergeCell ref="A178:A181"/>
+    <mergeCell ref="H154:H157"/>
+    <mergeCell ref="B194:B197"/>
+    <mergeCell ref="A174:A177"/>
+    <mergeCell ref="A194:A197"/>
+    <mergeCell ref="D118:D121"/>
+    <mergeCell ref="B126:B129"/>
+    <mergeCell ref="D182:D185"/>
+    <mergeCell ref="F182:F185"/>
+    <mergeCell ref="C74:C77"/>
+    <mergeCell ref="A110:A113"/>
+    <mergeCell ref="F162:F165"/>
+    <mergeCell ref="C166:C169"/>
+    <mergeCell ref="E6:E9"/>
+    <mergeCell ref="G6:G9"/>
+    <mergeCell ref="G62:G65"/>
+    <mergeCell ref="A154:A157"/>
+    <mergeCell ref="F190:F193"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="H190:H193"/>
+    <mergeCell ref="D30:D33"/>
+    <mergeCell ref="A106:A109"/>
+    <mergeCell ref="H14:H17"/>
+    <mergeCell ref="B54:B57"/>
+    <mergeCell ref="G42:G45"/>
+    <mergeCell ref="B94:B97"/>
+    <mergeCell ref="C126:C129"/>
+    <mergeCell ref="H122:H125"/>
+    <mergeCell ref="E126:E129"/>
+    <mergeCell ref="B102:B105"/>
+    <mergeCell ref="E190:E193"/>
+    <mergeCell ref="D158:D161"/>
+    <mergeCell ref="G190:G193"/>
+    <mergeCell ref="H74:H77"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="C50:C53"/>
+    <mergeCell ref="H46:H49"/>
+    <mergeCell ref="H26:H29"/>
+    <mergeCell ref="C42:C45"/>
+    <mergeCell ref="H38:H41"/>
+    <mergeCell ref="F74:F77"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="E42:E45"/>
+    <mergeCell ref="H130:H133"/>
+    <mergeCell ref="B106:B109"/>
+    <mergeCell ref="B170:B173"/>
+    <mergeCell ref="D170:D173"/>
+    <mergeCell ref="A86:A89"/>
+    <mergeCell ref="F138:F141"/>
+    <mergeCell ref="C142:C145"/>
+    <mergeCell ref="H138:H141"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="H34:H37"/>
+    <mergeCell ref="H162:H165"/>
+    <mergeCell ref="E138:E141"/>
+    <mergeCell ref="A118:A121"/>
+    <mergeCell ref="F114:F117"/>
+    <mergeCell ref="C118:C121"/>
+    <mergeCell ref="H114:H117"/>
+    <mergeCell ref="H70:H73"/>
+    <mergeCell ref="D66:D69"/>
+    <mergeCell ref="B186:B189"/>
+    <mergeCell ref="B142:B145"/>
+    <mergeCell ref="G138:G141"/>
+    <mergeCell ref="E174:E177"/>
+    <mergeCell ref="D142:D145"/>
+    <mergeCell ref="E26:E29"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="C34:C37"/>
+    <mergeCell ref="D10:D13"/>
+    <mergeCell ref="F10:F13"/>
+    <mergeCell ref="G14:G17"/>
+    <mergeCell ref="D18:D21"/>
+    <mergeCell ref="B178:B181"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="F66:F69"/>
+    <mergeCell ref="B74:B77"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="F38:F41"/>
+    <mergeCell ref="E162:E165"/>
+    <mergeCell ref="D130:D133"/>
+    <mergeCell ref="A134:A137"/>
+    <mergeCell ref="F130:F133"/>
+    <mergeCell ref="A126:A129"/>
+    <mergeCell ref="F106:F109"/>
+    <mergeCell ref="D194:D197"/>
+    <mergeCell ref="F134:F137"/>
+    <mergeCell ref="A198:A201"/>
+    <mergeCell ref="F194:F197"/>
+    <mergeCell ref="C198:C201"/>
+    <mergeCell ref="H194:H197"/>
+    <mergeCell ref="C110:C113"/>
+    <mergeCell ref="H18:H21"/>
+    <mergeCell ref="B154:B157"/>
+    <mergeCell ref="C174:C177"/>
+    <mergeCell ref="G46:G49"/>
+    <mergeCell ref="H106:H109"/>
     <mergeCell ref="A30:A33"/>
-    <mergeCell ref="C162:C165"/>
-    <mergeCell ref="B130:B133"/>
     <mergeCell ref="C30:C33"/>
-    <mergeCell ref="E38:E41"/>
     <mergeCell ref="A54:A57"/>
-    <mergeCell ref="D46:D49"/>
     <mergeCell ref="C54:C57"/>
-    <mergeCell ref="A74:A77"/>
+    <mergeCell ref="A90:A93"/>
+    <mergeCell ref="A146:A149"/>
+    <mergeCell ref="C146:C149"/>
+    <mergeCell ref="D126:D129"/>
+    <mergeCell ref="C94:C97"/>
+    <mergeCell ref="F126:F129"/>
+    <mergeCell ref="E94:E97"/>
+    <mergeCell ref="H182:H185"/>
+    <mergeCell ref="A186:A189"/>
+    <mergeCell ref="C186:C189"/>
+    <mergeCell ref="E142:E145"/>
+    <mergeCell ref="H82:H85"/>
+    <mergeCell ref="F118:F121"/>
+    <mergeCell ref="H118:H121"/>
+    <mergeCell ref="G2:G5"/>
+    <mergeCell ref="A138:A141"/>
+    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="E10:E13"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="B70:B73"/>
+    <mergeCell ref="G10:G13"/>
+    <mergeCell ref="G66:G69"/>
+    <mergeCell ref="D70:D73"/>
+    <mergeCell ref="F70:F73"/>
+    <mergeCell ref="D134:D137"/>
     <mergeCell ref="B38:B41"/>
+    <mergeCell ref="E158:E161"/>
     <mergeCell ref="F46:F49"/>
     <mergeCell ref="E74:E77"/>
     <mergeCell ref="B78:B81"/>
     <mergeCell ref="F42:F45"/>
-    <mergeCell ref="E50:E53"/>
-    <mergeCell ref="D82:D85"/>
-    <mergeCell ref="F82:F85"/>
-    <mergeCell ref="C86:C89"/>
-    <mergeCell ref="E130:E133"/>
-    <mergeCell ref="D54:D57"/>
-    <mergeCell ref="B134:B137"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="A118:A121"/>
-    <mergeCell ref="D198:D201"/>
-    <mergeCell ref="A90:A93"/>
-    <mergeCell ref="A146:A149"/>
-    <mergeCell ref="F198:F201"/>
-    <mergeCell ref="C146:C149"/>
-    <mergeCell ref="D174:D177"/>
-    <mergeCell ref="F174:F177"/>
-    <mergeCell ref="A178:A181"/>
-    <mergeCell ref="D126:D129"/>
-    <mergeCell ref="C94:C97"/>
-    <mergeCell ref="F126:F129"/>
-    <mergeCell ref="D166:D169"/>
-    <mergeCell ref="E94:E97"/>
-    <mergeCell ref="E90:E93"/>
-    <mergeCell ref="F110:F113"/>
-    <mergeCell ref="D150:D153"/>
-    <mergeCell ref="F150:F153"/>
-    <mergeCell ref="E158:E161"/>
-    <mergeCell ref="B166:B169"/>
-    <mergeCell ref="B118:B121"/>
-    <mergeCell ref="E154:E157"/>
-    <mergeCell ref="E110:E113"/>
-    <mergeCell ref="F94:F97"/>
-    <mergeCell ref="F98:F101"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="B158:B161"/>
-    <mergeCell ref="D78:D81"/>
-    <mergeCell ref="C2:C5"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="E2:E5"/>
-    <mergeCell ref="B186:B189"/>
-    <mergeCell ref="C82:C85"/>
-    <mergeCell ref="D102:D105"/>
-    <mergeCell ref="B142:B145"/>
-    <mergeCell ref="E174:E177"/>
-    <mergeCell ref="D142:D145"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="A150:A153"/>
-    <mergeCell ref="E26:E29"/>
-    <mergeCell ref="D98:D101"/>
-    <mergeCell ref="C66:C69"/>
-    <mergeCell ref="A102:A105"/>
-    <mergeCell ref="E66:E69"/>
-    <mergeCell ref="C102:C105"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="C34:C37"/>
-    <mergeCell ref="B194:B197"/>
-    <mergeCell ref="D10:D13"/>
-    <mergeCell ref="B90:B93"/>
-    <mergeCell ref="D50:D53"/>
-    <mergeCell ref="F10:F13"/>
-    <mergeCell ref="A94:A97"/>
-    <mergeCell ref="F146:F149"/>
-    <mergeCell ref="B122:B125"/>
-    <mergeCell ref="E150:E153"/>
-    <mergeCell ref="D178:D181"/>
-    <mergeCell ref="D34:D37"/>
-    <mergeCell ref="A182:A185"/>
-    <mergeCell ref="F178:F181"/>
-    <mergeCell ref="C42:C45"/>
-    <mergeCell ref="B18:B21"/>
-    <mergeCell ref="F34:F37"/>
-    <mergeCell ref="F74:F77"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="E42:E45"/>
-    <mergeCell ref="B106:B109"/>
-    <mergeCell ref="E186:E189"/>
-    <mergeCell ref="A194:A197"/>
-    <mergeCell ref="E30:E33"/>
-    <mergeCell ref="C70:C73"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="D2:D5"/>
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="C22:C25"/>
-    <mergeCell ref="E122:E125"/>
-    <mergeCell ref="F18:F21"/>
-    <mergeCell ref="B170:B173"/>
-    <mergeCell ref="E78:E81"/>
-    <mergeCell ref="A174:A177"/>
-    <mergeCell ref="D170:D173"/>
-    <mergeCell ref="F2:F5"/>
-    <mergeCell ref="B58:B61"/>
-    <mergeCell ref="E6:E9"/>
-    <mergeCell ref="C134:C137"/>
-    <mergeCell ref="C114:C117"/>
-    <mergeCell ref="A154:A157"/>
-    <mergeCell ref="F22:F25"/>
-    <mergeCell ref="E114:E117"/>
-    <mergeCell ref="E170:E173"/>
-    <mergeCell ref="F102:F105"/>
-    <mergeCell ref="E70:E73"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="C106:C109"/>
-    <mergeCell ref="C46:C49"/>
-    <mergeCell ref="F190:F193"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="C138:C141"/>
-    <mergeCell ref="C178:C181"/>
-    <mergeCell ref="E54:E57"/>
-    <mergeCell ref="D30:D33"/>
-    <mergeCell ref="E178:E181"/>
-    <mergeCell ref="D62:D65"/>
-    <mergeCell ref="D118:D121"/>
-    <mergeCell ref="F62:F65"/>
-    <mergeCell ref="E126:E129"/>
-    <mergeCell ref="C166:C169"/>
-    <mergeCell ref="B94:B97"/>
+    <mergeCell ref="G74:G77"/>
+    <mergeCell ref="B198:B201"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A130:A133"/>
+    <mergeCell ref="B110:B113"/>
+    <mergeCell ref="D110:D113"/>
+    <mergeCell ref="E146:E149"/>
+    <mergeCell ref="F166:F169"/>
     <mergeCell ref="C58:C61"/>
     <mergeCell ref="E58:E61"/>
-    <mergeCell ref="D90:D93"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="B102:B105"/>
-    <mergeCell ref="E138:E141"/>
-    <mergeCell ref="E190:E193"/>
-    <mergeCell ref="D158:D161"/>
-    <mergeCell ref="B98:B101"/>
-    <mergeCell ref="F114:F117"/>
-    <mergeCell ref="D154:D157"/>
-    <mergeCell ref="B198:B201"/>
-    <mergeCell ref="A106:A109"/>
-    <mergeCell ref="D14:D17"/>
-    <mergeCell ref="F14:F17"/>
-    <mergeCell ref="B174:B177"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="B126:B129"/>
-    <mergeCell ref="D182:D185"/>
-    <mergeCell ref="A130:A133"/>
-    <mergeCell ref="F182:F185"/>
-    <mergeCell ref="D38:D41"/>
-    <mergeCell ref="A82:A85"/>
-    <mergeCell ref="B110:B113"/>
-    <mergeCell ref="E106:E109"/>
-    <mergeCell ref="D110:D113"/>
-    <mergeCell ref="B54:B57"/>
-    <mergeCell ref="E146:E149"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="F166:F169"/>
-    <mergeCell ref="E198:E201"/>
-    <mergeCell ref="C74:C77"/>
-    <mergeCell ref="C126:C129"/>
-    <mergeCell ref="F162:F165"/>
-    <mergeCell ref="A110:A113"/>
-    <mergeCell ref="F26:F29"/>
-    <mergeCell ref="F154:F157"/>
-    <mergeCell ref="A158:A161"/>
-    <mergeCell ref="C118:C121"/>
     <mergeCell ref="D186:D189"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="C50:C53"/>
     <mergeCell ref="B82:B85"/>
-    <mergeCell ref="A86:A89"/>
-    <mergeCell ref="F138:F141"/>
-    <mergeCell ref="C142:C145"/>
     <mergeCell ref="F90:F93"/>
     <mergeCell ref="E118:E121"/>
-    <mergeCell ref="B10:B13"/>
-    <mergeCell ref="E46:E49"/>
-    <mergeCell ref="D66:D69"/>
-    <mergeCell ref="D106:D109"/>
     <mergeCell ref="B146:B149"/>
-    <mergeCell ref="F66:F69"/>
-    <mergeCell ref="D18:D21"/>
     <mergeCell ref="D146:D149"/>
     <mergeCell ref="E166:E169"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="B178:B181"/>
-    <mergeCell ref="E86:E89"/>
-    <mergeCell ref="B34:B37"/>
-    <mergeCell ref="B74:B77"/>
-    <mergeCell ref="A42:A45"/>
     <mergeCell ref="F50:F53"/>
-    <mergeCell ref="F38:F41"/>
-    <mergeCell ref="E162:E165"/>
-    <mergeCell ref="D130:D133"/>
-    <mergeCell ref="A134:A137"/>
-    <mergeCell ref="B162:B165"/>
-    <mergeCell ref="F130:F133"/>
-    <mergeCell ref="D74:D77"/>
-    <mergeCell ref="E134:E137"/>
-    <mergeCell ref="D138:D141"/>
-    <mergeCell ref="F54:F57"/>
-    <mergeCell ref="C158:C161"/>
-    <mergeCell ref="C194:C197"/>
     <mergeCell ref="C38:C41"/>
     <mergeCell ref="D58:D61"/>
     <mergeCell ref="A62:A65"/>
@@ -4380,173 +4486,67 @@
     <mergeCell ref="A122:A125"/>
     <mergeCell ref="C122:C125"/>
     <mergeCell ref="C78:C81"/>
-    <mergeCell ref="D42:D45"/>
-    <mergeCell ref="A186:A189"/>
-    <mergeCell ref="C186:C189"/>
-    <mergeCell ref="D94:D97"/>
-    <mergeCell ref="E142:E145"/>
-    <mergeCell ref="E194:E197"/>
-    <mergeCell ref="B150:B153"/>
-    <mergeCell ref="A114:A117"/>
-    <mergeCell ref="A170:A173"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="C170:C173"/>
-    <mergeCell ref="F78:F81"/>
-    <mergeCell ref="F118:F121"/>
-    <mergeCell ref="F158:F161"/>
-    <mergeCell ref="B190:B193"/>
-    <mergeCell ref="D194:D197"/>
-    <mergeCell ref="D6:D9"/>
-    <mergeCell ref="C26:C29"/>
-    <mergeCell ref="D190:D193"/>
-    <mergeCell ref="F6:F9"/>
-    <mergeCell ref="A138:A141"/>
-    <mergeCell ref="B86:B89"/>
-    <mergeCell ref="E82:E85"/>
-    <mergeCell ref="D86:D89"/>
-    <mergeCell ref="F86:F89"/>
-    <mergeCell ref="F142:F145"/>
-    <mergeCell ref="C10:C13"/>
-    <mergeCell ref="B62:B65"/>
-    <mergeCell ref="E10:E13"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="B70:B73"/>
-    <mergeCell ref="D70:D73"/>
-    <mergeCell ref="E98:E101"/>
-    <mergeCell ref="F70:F73"/>
-    <mergeCell ref="E34:E37"/>
-    <mergeCell ref="B182:B185"/>
-    <mergeCell ref="D134:D137"/>
-    <mergeCell ref="F134:F137"/>
-    <mergeCell ref="E62:E65"/>
-    <mergeCell ref="E22:E25"/>
-    <mergeCell ref="A198:A201"/>
-    <mergeCell ref="F194:F197"/>
-    <mergeCell ref="C198:C201"/>
-    <mergeCell ref="D122:D125"/>
-    <mergeCell ref="C90:C93"/>
-    <mergeCell ref="A126:A129"/>
-    <mergeCell ref="D162:D165"/>
-    <mergeCell ref="C130:C133"/>
-    <mergeCell ref="F122:F125"/>
-    <mergeCell ref="C182:C185"/>
-    <mergeCell ref="A142:A145"/>
-    <mergeCell ref="E182:E185"/>
-    <mergeCell ref="C110:C113"/>
-    <mergeCell ref="F106:F109"/>
-    <mergeCell ref="F186:F189"/>
-    <mergeCell ref="C150:C153"/>
-    <mergeCell ref="A190:A193"/>
-    <mergeCell ref="C190:C193"/>
+    <mergeCell ref="A182:A185"/>
+    <mergeCell ref="F178:F181"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="F34:F37"/>
+    <mergeCell ref="F2:F5"/>
+    <mergeCell ref="H2:H5"/>
+    <mergeCell ref="H94:H97"/>
+    <mergeCell ref="C114:C117"/>
+    <mergeCell ref="C70:C73"/>
+    <mergeCell ref="E114:E117"/>
+    <mergeCell ref="E170:E173"/>
+    <mergeCell ref="F102:F105"/>
+    <mergeCell ref="E70:E73"/>
+    <mergeCell ref="H66:H69"/>
+    <mergeCell ref="C106:C109"/>
+    <mergeCell ref="C178:C181"/>
+    <mergeCell ref="E178:E181"/>
+    <mergeCell ref="D62:D65"/>
+    <mergeCell ref="F62:F65"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="H90:H93"/>
+    <mergeCell ref="G118:G121"/>
+    <mergeCell ref="G182:G185"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="H158:H161"/>
+    <mergeCell ref="E50:E53"/>
+    <mergeCell ref="C86:C89"/>
+    <mergeCell ref="G50:G53"/>
+    <mergeCell ref="D54:D57"/>
+    <mergeCell ref="B122:B125"/>
+    <mergeCell ref="E150:E153"/>
+    <mergeCell ref="D178:D181"/>
+    <mergeCell ref="D34:D37"/>
+    <mergeCell ref="G134:G137"/>
+    <mergeCell ref="H166:H169"/>
+    <mergeCell ref="E110:E113"/>
+    <mergeCell ref="D78:D81"/>
     <mergeCell ref="B114:B117"/>
     <mergeCell ref="D114:D117"/>
-    <mergeCell ref="B154:B157"/>
-    <mergeCell ref="C174:C177"/>
     <mergeCell ref="F170:F173"/>
-    <mergeCell ref="B138:B141"/>
-    <mergeCell ref="C6:C9"/>
-    <mergeCell ref="C62:C65"/>
+    <mergeCell ref="H170:H173"/>
+    <mergeCell ref="G166:G169"/>
+    <mergeCell ref="D150:D153"/>
     <mergeCell ref="A98:A101"/>
-    <mergeCell ref="G2:G5"/>
-    <mergeCell ref="H2:H5"/>
-    <mergeCell ref="G6:G9"/>
-    <mergeCell ref="H6:H9"/>
-    <mergeCell ref="G10:G13"/>
-    <mergeCell ref="H10:H13"/>
-    <mergeCell ref="G14:G17"/>
-    <mergeCell ref="H14:H17"/>
-    <mergeCell ref="G18:G21"/>
-    <mergeCell ref="H18:H21"/>
-    <mergeCell ref="G22:G25"/>
-    <mergeCell ref="H22:H25"/>
+    <mergeCell ref="F150:F153"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="F94:F97"/>
     <mergeCell ref="G26:G29"/>
-    <mergeCell ref="H26:H29"/>
-    <mergeCell ref="G30:G33"/>
-    <mergeCell ref="H30:H33"/>
-    <mergeCell ref="G34:G37"/>
-    <mergeCell ref="H34:H37"/>
-    <mergeCell ref="G38:G41"/>
-    <mergeCell ref="H38:H41"/>
-    <mergeCell ref="G42:G45"/>
-    <mergeCell ref="H42:H45"/>
-    <mergeCell ref="G46:G49"/>
-    <mergeCell ref="H46:H49"/>
-    <mergeCell ref="G50:G53"/>
-    <mergeCell ref="H50:H53"/>
-    <mergeCell ref="G54:G57"/>
-    <mergeCell ref="H54:H57"/>
-    <mergeCell ref="G58:G61"/>
-    <mergeCell ref="H58:H61"/>
-    <mergeCell ref="G62:G65"/>
-    <mergeCell ref="H62:H65"/>
-    <mergeCell ref="G66:G69"/>
-    <mergeCell ref="H66:H69"/>
-    <mergeCell ref="G70:G73"/>
-    <mergeCell ref="H70:H73"/>
-    <mergeCell ref="G74:G77"/>
-    <mergeCell ref="H74:H77"/>
-    <mergeCell ref="G78:G81"/>
-    <mergeCell ref="H78:H81"/>
-    <mergeCell ref="G82:G85"/>
-    <mergeCell ref="H82:H85"/>
-    <mergeCell ref="G86:G89"/>
-    <mergeCell ref="H86:H89"/>
-    <mergeCell ref="G90:G93"/>
-    <mergeCell ref="H90:H93"/>
-    <mergeCell ref="G94:G97"/>
-    <mergeCell ref="H94:H97"/>
-    <mergeCell ref="G98:G101"/>
-    <mergeCell ref="H98:H101"/>
+    <mergeCell ref="C82:C85"/>
+    <mergeCell ref="D102:D105"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="B66:B69"/>
+    <mergeCell ref="C154:C157"/>
+    <mergeCell ref="C98:C101"/>
+    <mergeCell ref="E102:E105"/>
     <mergeCell ref="G102:G105"/>
-    <mergeCell ref="H102:H105"/>
-    <mergeCell ref="G106:G109"/>
-    <mergeCell ref="H106:H109"/>
-    <mergeCell ref="G110:G113"/>
-    <mergeCell ref="H110:H113"/>
-    <mergeCell ref="G114:G117"/>
-    <mergeCell ref="H114:H117"/>
-    <mergeCell ref="G118:G121"/>
-    <mergeCell ref="H118:H121"/>
-    <mergeCell ref="G122:G125"/>
-    <mergeCell ref="H122:H125"/>
-    <mergeCell ref="G126:G129"/>
-    <mergeCell ref="H126:H129"/>
-    <mergeCell ref="G130:G133"/>
-    <mergeCell ref="H130:H133"/>
-    <mergeCell ref="G134:G137"/>
-    <mergeCell ref="H134:H137"/>
-    <mergeCell ref="G138:G141"/>
-    <mergeCell ref="H138:H141"/>
-    <mergeCell ref="G142:G145"/>
-    <mergeCell ref="H142:H145"/>
-    <mergeCell ref="G146:G149"/>
-    <mergeCell ref="H146:H149"/>
-    <mergeCell ref="G150:G153"/>
-    <mergeCell ref="H150:H153"/>
-    <mergeCell ref="G154:G157"/>
-    <mergeCell ref="H154:H157"/>
-    <mergeCell ref="G158:G161"/>
-    <mergeCell ref="H158:H161"/>
-    <mergeCell ref="G162:G165"/>
-    <mergeCell ref="H162:H165"/>
-    <mergeCell ref="G166:G169"/>
-    <mergeCell ref="H166:H169"/>
-    <mergeCell ref="G170:G173"/>
-    <mergeCell ref="H170:H173"/>
-    <mergeCell ref="G174:G177"/>
-    <mergeCell ref="H174:H177"/>
-    <mergeCell ref="G178:G181"/>
-    <mergeCell ref="H178:H181"/>
-    <mergeCell ref="G182:G185"/>
-    <mergeCell ref="H182:H185"/>
-    <mergeCell ref="G186:G189"/>
-    <mergeCell ref="H186:H189"/>
-    <mergeCell ref="G190:G193"/>
-    <mergeCell ref="H190:H193"/>
-    <mergeCell ref="G194:G197"/>
-    <mergeCell ref="H194:H197"/>
-    <mergeCell ref="G198:G201"/>
-    <mergeCell ref="H198:H201"/>
+    <mergeCell ref="A162:A165"/>
+    <mergeCell ref="F30:F33"/>
+    <mergeCell ref="C162:C165"/>
+    <mergeCell ref="B130:B133"/>
+    <mergeCell ref="D46:D49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
test: expand test case coverage for assignment 1
</commit_message>
<xml_diff>
--- a/IT23622814.xlsx
+++ b/IT23622814.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT23622814\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_5D85D03E51298B94020683252B36F527575834AB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82670C50-C07A-4352-BDDF-4788C54ED437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="722" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="297">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -908,6 +908,9 @@
   </si>
   <si>
     <t>Rationale: Input includes a specific website link identifier: 'www.news.lk'.</t>
+  </si>
+  <si>
+    <t>Greetings</t>
   </si>
 </sst>
 </file>
@@ -1013,21 +1016,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1351,25 +1354,25 @@
       <c r="A2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="2" t="s">
+      <c r="F2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="5" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1407,25 +1410,25 @@
       <c r="A6" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="2" t="s">
+      <c r="F6" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="5" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1463,25 +1466,25 @@
       <c r="A10" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="2" t="s">
+      <c r="F10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="5" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1519,25 +1522,25 @@
       <c r="A14" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="2" t="s">
+      <c r="F14" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="H14" s="5" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1575,23 +1578,25 @@
       <c r="A18" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="F18" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2" t="s">
+      <c r="F18" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>296</v>
+      </c>
+      <c r="H18" s="5" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1629,25 +1634,25 @@
       <c r="A22" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="E22" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="F22" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" s="2" t="s">
+      <c r="F22" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="H22" s="2" t="s">
+      <c r="H22" s="5" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1685,25 +1690,25 @@
       <c r="A26" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="E26" s="8" t="s">
+      <c r="E26" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="F26" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G26" s="2" t="s">
+      <c r="F26" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="H26" s="2" t="s">
+      <c r="H26" s="5" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1741,25 +1746,25 @@
       <c r="A30" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="C30" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="E30" s="8" t="s">
+      <c r="E30" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="F30" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G30" s="2" t="s">
+      <c r="F30" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="H30" s="2" t="s">
+      <c r="H30" s="5" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1797,25 +1802,25 @@
       <c r="A34" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="D34" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="E34" s="8" t="s">
+      <c r="E34" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="F34" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G34" s="2" t="s">
+      <c r="F34" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G34" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="H34" s="2" t="s">
+      <c r="H34" s="5" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1853,25 +1858,25 @@
       <c r="A38" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="C38" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="D38" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="E38" s="8" t="s">
+      <c r="E38" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="F38" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G38" s="2" t="s">
+      <c r="F38" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G38" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="H38" s="2" t="s">
+      <c r="H38" s="5" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1909,25 +1914,25 @@
       <c r="A42" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="C42" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D42" s="7" t="s">
+      <c r="D42" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E42" s="8" t="s">
+      <c r="E42" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="F42" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G42" s="2" t="s">
+      <c r="F42" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G42" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="H42" s="2" t="s">
+      <c r="H42" s="5" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1965,25 +1970,25 @@
       <c r="A46" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B46" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C46" s="5" t="s">
+      <c r="C46" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="D46" s="7" t="s">
+      <c r="D46" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E46" s="8" t="s">
+      <c r="E46" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="F46" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G46" s="2" t="s">
+      <c r="F46" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G46" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="H46" s="2" t="s">
+      <c r="H46" s="5" t="s">
         <v>76</v>
       </c>
     </row>
@@ -2021,25 +2026,25 @@
       <c r="A50" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B50" s="2" t="s">
+      <c r="B50" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C50" s="5" t="s">
+      <c r="C50" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D50" s="7" t="s">
+      <c r="D50" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E50" s="8" t="s">
+      <c r="E50" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="F50" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G50" s="2" t="s">
+      <c r="F50" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G50" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="H50" s="2" t="s">
+      <c r="H50" s="5" t="s">
         <v>82</v>
       </c>
     </row>
@@ -2077,25 +2082,25 @@
       <c r="A54" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="B54" s="2" t="s">
+      <c r="B54" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C54" s="5" t="s">
+      <c r="C54" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="D54" s="5" t="s">
+      <c r="D54" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E54" s="5" t="s">
+      <c r="E54" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="F54" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G54" s="5" t="s">
+      <c r="F54" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G54" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="H54" s="5" t="s">
+      <c r="H54" s="2" t="s">
         <v>87</v>
       </c>
     </row>
@@ -2133,25 +2138,25 @@
       <c r="A58" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="B58" s="2" t="s">
+      <c r="B58" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C58" s="5" t="s">
+      <c r="C58" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="D58" s="5" t="s">
+      <c r="D58" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="E58" s="5" t="s">
+      <c r="E58" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="F58" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G58" s="5" t="s">
+      <c r="F58" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G58" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="H58" s="5" t="s">
+      <c r="H58" s="2" t="s">
         <v>93</v>
       </c>
     </row>
@@ -2189,25 +2194,25 @@
       <c r="A62" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="B62" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C62" s="5" t="s">
+      <c r="C62" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D62" s="5" t="s">
+      <c r="D62" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="E62" s="5" t="s">
+      <c r="E62" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="F62" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G62" s="5" t="s">
+      <c r="F62" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G62" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="H62" s="5" t="s">
+      <c r="H62" s="2" t="s">
         <v>99</v>
       </c>
     </row>
@@ -2245,25 +2250,25 @@
       <c r="A66" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="B66" s="2" t="s">
+      <c r="B66" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C66" s="5" t="s">
+      <c r="C66" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="D66" s="5" t="s">
+      <c r="D66" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E66" s="5" t="s">
+      <c r="E66" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="F66" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G66" s="5" t="s">
+      <c r="F66" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G66" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="H66" s="5" t="s">
+      <c r="H66" s="2" t="s">
         <v>105</v>
       </c>
     </row>
@@ -2301,25 +2306,25 @@
       <c r="A70" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="B70" s="2" t="s">
+      <c r="B70" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C70" s="5" t="s">
+      <c r="C70" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="D70" s="5" t="s">
+      <c r="D70" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="E70" s="5" t="s">
+      <c r="E70" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="F70" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G70" s="5" t="s">
+      <c r="F70" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G70" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="H70" s="5" t="s">
+      <c r="H70" s="2" t="s">
         <v>111</v>
       </c>
     </row>
@@ -2357,25 +2362,25 @@
       <c r="A74" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="B74" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C74" s="5" t="s">
+      <c r="C74" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D74" s="5" t="s">
+      <c r="D74" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="E74" s="5" t="s">
+      <c r="E74" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="F74" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G74" s="5" t="s">
+      <c r="F74" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G74" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="H74" s="5" t="s">
+      <c r="H74" s="2" t="s">
         <v>117</v>
       </c>
     </row>
@@ -2413,25 +2418,25 @@
       <c r="A78" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="B78" s="2" t="s">
+      <c r="B78" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C78" s="5" t="s">
+      <c r="C78" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="D78" s="5" t="s">
+      <c r="D78" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="E78" s="5" t="s">
+      <c r="E78" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="F78" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G78" s="5" t="s">
+      <c r="F78" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G78" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="H78" s="5" t="s">
+      <c r="H78" s="2" t="s">
         <v>123</v>
       </c>
     </row>
@@ -2469,25 +2474,25 @@
       <c r="A82" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="B82" s="2" t="s">
+      <c r="B82" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C82" s="5" t="s">
+      <c r="C82" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="D82" s="5" t="s">
+      <c r="D82" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="E82" s="5" t="s">
+      <c r="E82" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="F82" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G82" s="5" t="s">
+      <c r="F82" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G82" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="H82" s="5" t="s">
+      <c r="H82" s="2" t="s">
         <v>129</v>
       </c>
     </row>
@@ -2525,25 +2530,25 @@
       <c r="A86" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="B86" s="2" t="s">
+      <c r="B86" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C86" s="5" t="s">
+      <c r="C86" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="D86" s="5" t="s">
+      <c r="D86" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="E86" s="5" t="s">
+      <c r="E86" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="F86" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G86" s="5" t="s">
+      <c r="F86" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G86" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="H86" s="5" t="s">
+      <c r="H86" s="2" t="s">
         <v>135</v>
       </c>
     </row>
@@ -2581,25 +2586,25 @@
       <c r="A90" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="B90" s="2" t="s">
+      <c r="B90" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C90" s="5" t="s">
+      <c r="C90" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="D90" s="5" t="s">
+      <c r="D90" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="E90" s="5" t="s">
+      <c r="E90" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="F90" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G90" s="5" t="s">
+      <c r="F90" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G90" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="H90" s="5" t="s">
+      <c r="H90" s="2" t="s">
         <v>141</v>
       </c>
     </row>
@@ -2637,25 +2642,25 @@
       <c r="A94" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="B94" s="2" t="s">
+      <c r="B94" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C94" s="5" t="s">
+      <c r="C94" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="D94" s="5" t="s">
+      <c r="D94" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="E94" s="5" t="s">
+      <c r="E94" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="F94" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G94" s="5" t="s">
+      <c r="F94" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G94" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="H94" s="5" t="s">
+      <c r="H94" s="2" t="s">
         <v>146</v>
       </c>
     </row>
@@ -2693,25 +2698,25 @@
       <c r="A98" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="B98" s="2" t="s">
+      <c r="B98" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C98" s="5" t="s">
+      <c r="C98" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="D98" s="5" t="s">
+      <c r="D98" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="E98" s="5" t="s">
+      <c r="E98" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="F98" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G98" s="5" t="s">
+      <c r="F98" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G98" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="H98" s="5" t="s">
+      <c r="H98" s="2" t="s">
         <v>152</v>
       </c>
     </row>
@@ -2749,25 +2754,25 @@
       <c r="A102" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="B102" s="2" t="s">
+      <c r="B102" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C102" s="5" t="s">
+      <c r="C102" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="D102" s="5" t="s">
+      <c r="D102" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="E102" s="5" t="s">
+      <c r="E102" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="F102" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G102" s="5" t="s">
+      <c r="F102" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G102" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="H102" s="5" t="s">
+      <c r="H102" s="2" t="s">
         <v>158</v>
       </c>
     </row>
@@ -2805,25 +2810,25 @@
       <c r="A106" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="B106" s="2" t="s">
+      <c r="B106" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C106" s="5" t="s">
+      <c r="C106" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="D106" s="5" t="s">
+      <c r="D106" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="E106" s="5" t="s">
+      <c r="E106" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="F106" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G106" s="5" t="s">
+      <c r="F106" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G106" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="H106" s="5" t="s">
+      <c r="H106" s="2" t="s">
         <v>164</v>
       </c>
     </row>
@@ -2861,25 +2866,25 @@
       <c r="A110" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="B110" s="2" t="s">
+      <c r="B110" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C110" s="5" t="s">
+      <c r="C110" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="D110" s="5" t="s">
+      <c r="D110" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="E110" s="5" t="s">
+      <c r="E110" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="F110" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G110" s="5" t="s">
+      <c r="F110" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G110" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="H110" s="5" t="s">
+      <c r="H110" s="2" t="s">
         <v>169</v>
       </c>
     </row>
@@ -2917,25 +2922,25 @@
       <c r="A114" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="B114" s="2" t="s">
+      <c r="B114" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C114" s="5" t="s">
+      <c r="C114" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="D114" s="5" t="s">
+      <c r="D114" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="E114" s="5" t="s">
+      <c r="E114" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="F114" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G114" s="5" t="s">
+      <c r="F114" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G114" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="H114" s="5" t="s">
+      <c r="H114" s="2" t="s">
         <v>175</v>
       </c>
     </row>
@@ -2973,25 +2978,25 @@
       <c r="A118" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="B118" s="2" t="s">
+      <c r="B118" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C118" s="5" t="s">
+      <c r="C118" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="D118" s="5" t="s">
+      <c r="D118" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E118" s="5" t="s">
+      <c r="E118" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="F118" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G118" s="5" t="s">
+      <c r="F118" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G118" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="H118" s="5" t="s">
+      <c r="H118" s="2" t="s">
         <v>180</v>
       </c>
     </row>
@@ -3029,25 +3034,25 @@
       <c r="A122" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="B122" s="2" t="s">
+      <c r="B122" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C122" s="5" t="s">
+      <c r="C122" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="D122" s="5" t="s">
+      <c r="D122" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="E122" s="5" t="s">
+      <c r="E122" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="F122" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G122" s="5" t="s">
+      <c r="F122" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G122" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="H122" s="5" t="s">
+      <c r="H122" s="2" t="s">
         <v>186</v>
       </c>
     </row>
@@ -3085,25 +3090,25 @@
       <c r="A126" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="B126" s="2" t="s">
+      <c r="B126" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C126" s="5" t="s">
+      <c r="C126" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="D126" s="5" t="s">
+      <c r="D126" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="E126" s="5" t="s">
+      <c r="E126" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="F126" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G126" s="5" t="s">
+      <c r="F126" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G126" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="H126" s="5" t="s">
+      <c r="H126" s="2" t="s">
         <v>192</v>
       </c>
     </row>
@@ -3141,25 +3146,25 @@
       <c r="A130" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="B130" s="2" t="s">
+      <c r="B130" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C130" s="5" t="s">
+      <c r="C130" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="D130" s="5" t="s">
+      <c r="D130" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="E130" s="5" t="s">
+      <c r="E130" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="F130" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G130" s="5" t="s">
+      <c r="F130" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G130" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="H130" s="5" t="s">
+      <c r="H130" s="2" t="s">
         <v>198</v>
       </c>
     </row>
@@ -3197,25 +3202,25 @@
       <c r="A134" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="B134" s="2" t="s">
+      <c r="B134" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C134" s="5" t="s">
+      <c r="C134" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="D134" s="5" t="s">
+      <c r="D134" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="E134" s="5" t="s">
+      <c r="E134" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="F134" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G134" s="5" t="s">
+      <c r="F134" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G134" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="H134" s="5" t="s">
+      <c r="H134" s="2" t="s">
         <v>203</v>
       </c>
     </row>
@@ -3253,25 +3258,25 @@
       <c r="A138" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="B138" s="2" t="s">
+      <c r="B138" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C138" s="5" t="s">
+      <c r="C138" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="D138" s="5" t="s">
+      <c r="D138" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="E138" s="5" t="s">
+      <c r="E138" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="F138" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G138" s="5" t="s">
+      <c r="F138" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G138" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="H138" s="5" t="s">
+      <c r="H138" s="2" t="s">
         <v>209</v>
       </c>
     </row>
@@ -3309,25 +3314,25 @@
       <c r="A142" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="B142" s="2" t="s">
+      <c r="B142" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C142" s="5" t="s">
+      <c r="C142" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="D142" s="5" t="s">
+      <c r="D142" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="E142" s="5" t="s">
+      <c r="E142" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="F142" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G142" s="5" t="s">
+      <c r="F142" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G142" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="H142" s="5" t="s">
+      <c r="H142" s="2" t="s">
         <v>215</v>
       </c>
     </row>
@@ -3365,25 +3370,25 @@
       <c r="A146" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="B146" s="2" t="s">
+      <c r="B146" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C146" s="5" t="s">
+      <c r="C146" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="D146" s="5" t="s">
+      <c r="D146" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="E146" s="5" t="s">
+      <c r="E146" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="F146" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G146" s="5" t="s">
+      <c r="F146" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G146" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="H146" s="5" t="s">
+      <c r="H146" s="2" t="s">
         <v>221</v>
       </c>
     </row>
@@ -3421,25 +3426,25 @@
       <c r="A150" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="B150" s="2" t="s">
+      <c r="B150" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C150" s="5" t="s">
+      <c r="C150" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="D150" s="5" t="s">
+      <c r="D150" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="E150" s="5" t="s">
+      <c r="E150" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="F150" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G150" s="5" t="s">
+      <c r="F150" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G150" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="H150" s="5" t="s">
+      <c r="H150" s="2" t="s">
         <v>227</v>
       </c>
     </row>
@@ -3477,25 +3482,25 @@
       <c r="A154" s="6" t="s">
         <v>228</v>
       </c>
-      <c r="B154" s="2" t="s">
+      <c r="B154" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C154" s="5" t="s">
+      <c r="C154" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="D154" s="5" t="s">
+      <c r="D154" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="E154" s="5" t="s">
+      <c r="E154" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="F154" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G154" s="5" t="s">
+      <c r="F154" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G154" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="H154" s="5" t="s">
+      <c r="H154" s="2" t="s">
         <v>233</v>
       </c>
     </row>
@@ -3533,25 +3538,25 @@
       <c r="A158" s="6" t="s">
         <v>234</v>
       </c>
-      <c r="B158" s="2" t="s">
+      <c r="B158" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C158" s="5" t="s">
+      <c r="C158" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="D158" s="5" t="s">
+      <c r="D158" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="E158" s="5" t="s">
+      <c r="E158" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="F158" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G158" s="5" t="s">
+      <c r="F158" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G158" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="H158" s="5" t="s">
+      <c r="H158" s="2" t="s">
         <v>239</v>
       </c>
     </row>
@@ -3589,25 +3594,25 @@
       <c r="A162" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="B162" s="2" t="s">
+      <c r="B162" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C162" s="5" t="s">
+      <c r="C162" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="D162" s="5" t="s">
+      <c r="D162" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="E162" s="5" t="s">
+      <c r="E162" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="F162" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G162" s="5" t="s">
+      <c r="F162" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G162" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="H162" s="5" t="s">
+      <c r="H162" s="2" t="s">
         <v>245</v>
       </c>
     </row>
@@ -3645,25 +3650,25 @@
       <c r="A166" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="B166" s="2" t="s">
+      <c r="B166" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C166" s="5" t="s">
+      <c r="C166" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="D166" s="5" t="s">
+      <c r="D166" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="E166" s="5" t="s">
+      <c r="E166" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="F166" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G166" s="5" t="s">
+      <c r="F166" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G166" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="H166" s="5" t="s">
+      <c r="H166" s="2" t="s">
         <v>251</v>
       </c>
     </row>
@@ -3701,25 +3706,25 @@
       <c r="A170" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="B170" s="2" t="s">
+      <c r="B170" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C170" s="5" t="s">
+      <c r="C170" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="D170" s="5" t="s">
+      <c r="D170" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="E170" s="5" t="s">
+      <c r="E170" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="F170" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G170" s="5" t="s">
+      <c r="F170" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G170" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="H170" s="5" t="s">
+      <c r="H170" s="2" t="s">
         <v>257</v>
       </c>
     </row>
@@ -3757,25 +3762,25 @@
       <c r="A174" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="B174" s="2" t="s">
+      <c r="B174" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C174" s="5" t="s">
+      <c r="C174" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="D174" s="5" t="s">
+      <c r="D174" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="E174" s="5" t="s">
+      <c r="E174" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="F174" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G174" s="5" t="s">
+      <c r="F174" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G174" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="H174" s="5" t="s">
+      <c r="H174" s="2" t="s">
         <v>262</v>
       </c>
     </row>
@@ -3813,25 +3818,25 @@
       <c r="A178" s="6" t="s">
         <v>263</v>
       </c>
-      <c r="B178" s="2" t="s">
+      <c r="B178" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C178" s="5" t="s">
+      <c r="C178" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="D178" s="5" t="s">
+      <c r="D178" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="E178" s="5" t="s">
+      <c r="E178" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="F178" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G178" s="5" t="s">
+      <c r="F178" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G178" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="H178" s="5" t="s">
+      <c r="H178" s="2" t="s">
         <v>268</v>
       </c>
     </row>
@@ -3869,25 +3874,25 @@
       <c r="A182" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="B182" s="2" t="s">
+      <c r="B182" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C182" s="5" t="s">
+      <c r="C182" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="D182" s="5" t="s">
+      <c r="D182" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="E182" s="5" t="s">
+      <c r="E182" s="2" t="s">
         <v>272</v>
       </c>
-      <c r="F182" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G182" s="5" t="s">
+      <c r="F182" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G182" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="H182" s="5" t="s">
+      <c r="H182" s="2" t="s">
         <v>273</v>
       </c>
     </row>
@@ -3925,25 +3930,25 @@
       <c r="A186" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="B186" s="2" t="s">
+      <c r="B186" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C186" s="5" t="s">
+      <c r="C186" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="D186" s="5" t="s">
+      <c r="D186" s="2" t="s">
         <v>276</v>
       </c>
-      <c r="E186" s="5" t="s">
+      <c r="E186" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="F186" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G186" s="5" t="s">
+      <c r="F186" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G186" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="H186" s="5" t="s">
+      <c r="H186" s="2" t="s">
         <v>279</v>
       </c>
     </row>
@@ -3981,25 +3986,25 @@
       <c r="A190" s="6" t="s">
         <v>280</v>
       </c>
-      <c r="B190" s="2" t="s">
+      <c r="B190" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C190" s="5" t="s">
+      <c r="C190" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="D190" s="5" t="s">
+      <c r="D190" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="E190" s="5" t="s">
+      <c r="E190" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="F190" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G190" s="5" t="s">
+      <c r="F190" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G190" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="H190" s="5" t="s">
+      <c r="H190" s="2" t="s">
         <v>284</v>
       </c>
     </row>
@@ -4037,25 +4042,25 @@
       <c r="A194" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="B194" s="2" t="s">
+      <c r="B194" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C194" s="5" t="s">
+      <c r="C194" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="D194" s="5" t="s">
+      <c r="D194" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="E194" s="5" t="s">
+      <c r="E194" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="F194" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G194" s="5" t="s">
+      <c r="F194" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G194" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="H194" s="5" t="s">
+      <c r="H194" s="2" t="s">
         <v>289</v>
       </c>
     </row>
@@ -4093,25 +4098,25 @@
       <c r="A198" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="B198" s="2" t="s">
+      <c r="B198" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C198" s="5" t="s">
+      <c r="C198" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="D198" s="5" t="s">
+      <c r="D198" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="E198" s="5" t="s">
+      <c r="E198" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="F198" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G198" s="5" t="s">
+      <c r="F198" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G198" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="H198" s="5" t="s">
+      <c r="H198" s="2" t="s">
         <v>295</v>
       </c>
     </row>
@@ -4147,57 +4152,310 @@
     </row>
   </sheetData>
   <mergeCells count="400">
-    <mergeCell ref="C6:C9"/>
-    <mergeCell ref="C62:C65"/>
-    <mergeCell ref="E62:E65"/>
-    <mergeCell ref="H6:H9"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="H98:H101"/>
-    <mergeCell ref="A66:A69"/>
-    <mergeCell ref="B98:B101"/>
-    <mergeCell ref="D154:D157"/>
-    <mergeCell ref="F154:F157"/>
-    <mergeCell ref="A158:A161"/>
-    <mergeCell ref="G174:G177"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="E46:E49"/>
-    <mergeCell ref="D106:D109"/>
-    <mergeCell ref="A26:A29"/>
-    <mergeCell ref="E86:E89"/>
-    <mergeCell ref="B162:B165"/>
-    <mergeCell ref="G150:G153"/>
-    <mergeCell ref="G94:G97"/>
-    <mergeCell ref="H126:H129"/>
-    <mergeCell ref="G158:G161"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="D22:D25"/>
-    <mergeCell ref="F78:F81"/>
-    <mergeCell ref="H78:H81"/>
-    <mergeCell ref="B86:B89"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="G58:G61"/>
-    <mergeCell ref="A150:A153"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="H186:H189"/>
-    <mergeCell ref="D26:D29"/>
-    <mergeCell ref="D82:D85"/>
-    <mergeCell ref="F82:F85"/>
-    <mergeCell ref="H30:H33"/>
-    <mergeCell ref="B90:B93"/>
-    <mergeCell ref="A94:A97"/>
-    <mergeCell ref="F146:F149"/>
-    <mergeCell ref="H146:H149"/>
-    <mergeCell ref="G126:G129"/>
-    <mergeCell ref="H10:H13"/>
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="H58:H61"/>
-    <mergeCell ref="C22:C25"/>
-    <mergeCell ref="E122:E125"/>
-    <mergeCell ref="E78:E81"/>
-    <mergeCell ref="G122:G125"/>
-    <mergeCell ref="G78:G81"/>
-    <mergeCell ref="C134:C137"/>
-    <mergeCell ref="E186:E189"/>
+    <mergeCell ref="A162:A165"/>
+    <mergeCell ref="F30:F33"/>
+    <mergeCell ref="C162:C165"/>
+    <mergeCell ref="B130:B133"/>
+    <mergeCell ref="D46:D49"/>
+    <mergeCell ref="A98:A101"/>
+    <mergeCell ref="F150:F153"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="F94:F97"/>
+    <mergeCell ref="G26:G29"/>
+    <mergeCell ref="C82:C85"/>
+    <mergeCell ref="D102:D105"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="B66:B69"/>
+    <mergeCell ref="C98:C101"/>
+    <mergeCell ref="E102:E105"/>
+    <mergeCell ref="G102:G105"/>
+    <mergeCell ref="H2:H5"/>
+    <mergeCell ref="H94:H97"/>
+    <mergeCell ref="C114:C117"/>
+    <mergeCell ref="C70:C73"/>
+    <mergeCell ref="E114:E117"/>
+    <mergeCell ref="E170:E173"/>
+    <mergeCell ref="F102:F105"/>
+    <mergeCell ref="E70:E73"/>
+    <mergeCell ref="H66:H69"/>
+    <mergeCell ref="C106:C109"/>
+    <mergeCell ref="D62:D65"/>
+    <mergeCell ref="F62:F65"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="H90:H93"/>
+    <mergeCell ref="G118:G121"/>
+    <mergeCell ref="H158:H161"/>
+    <mergeCell ref="E50:E53"/>
+    <mergeCell ref="C86:C89"/>
+    <mergeCell ref="G50:G53"/>
+    <mergeCell ref="D54:D57"/>
+    <mergeCell ref="E150:E153"/>
+    <mergeCell ref="D34:D37"/>
+    <mergeCell ref="G134:G137"/>
+    <mergeCell ref="H166:H169"/>
+    <mergeCell ref="B198:B201"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A130:A133"/>
+    <mergeCell ref="B110:B113"/>
+    <mergeCell ref="D110:D113"/>
+    <mergeCell ref="E146:E149"/>
+    <mergeCell ref="F166:F169"/>
+    <mergeCell ref="C58:C61"/>
+    <mergeCell ref="E58:E61"/>
+    <mergeCell ref="D186:D189"/>
+    <mergeCell ref="B82:B85"/>
+    <mergeCell ref="F90:F93"/>
+    <mergeCell ref="E118:E121"/>
+    <mergeCell ref="B146:B149"/>
+    <mergeCell ref="D146:D149"/>
+    <mergeCell ref="E166:E169"/>
+    <mergeCell ref="F50:F53"/>
+    <mergeCell ref="C38:C41"/>
+    <mergeCell ref="D58:D61"/>
+    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="F58:F61"/>
+    <mergeCell ref="A122:A125"/>
+    <mergeCell ref="C122:C125"/>
+    <mergeCell ref="C78:C81"/>
+    <mergeCell ref="G2:G5"/>
+    <mergeCell ref="A138:A141"/>
+    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="E10:E13"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="B70:B73"/>
+    <mergeCell ref="G10:G13"/>
+    <mergeCell ref="G66:G69"/>
+    <mergeCell ref="D70:D73"/>
+    <mergeCell ref="F70:F73"/>
+    <mergeCell ref="D134:D137"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="F46:F49"/>
+    <mergeCell ref="E74:E77"/>
+    <mergeCell ref="B78:B81"/>
+    <mergeCell ref="F42:F45"/>
+    <mergeCell ref="G74:G77"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="F34:F37"/>
+    <mergeCell ref="F2:F5"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="B122:B125"/>
+    <mergeCell ref="E110:E113"/>
+    <mergeCell ref="D78:D81"/>
+    <mergeCell ref="D194:D197"/>
+    <mergeCell ref="F134:F137"/>
+    <mergeCell ref="A198:A201"/>
+    <mergeCell ref="F194:F197"/>
+    <mergeCell ref="C198:C201"/>
+    <mergeCell ref="H194:H197"/>
+    <mergeCell ref="C110:C113"/>
+    <mergeCell ref="H18:H21"/>
+    <mergeCell ref="B154:B157"/>
+    <mergeCell ref="C174:C177"/>
+    <mergeCell ref="G46:G49"/>
+    <mergeCell ref="H106:H109"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="C30:C33"/>
+    <mergeCell ref="A54:A57"/>
+    <mergeCell ref="C54:C57"/>
+    <mergeCell ref="A90:A93"/>
+    <mergeCell ref="A146:A149"/>
+    <mergeCell ref="C146:C149"/>
+    <mergeCell ref="D126:D129"/>
+    <mergeCell ref="C94:C97"/>
+    <mergeCell ref="F126:F129"/>
+    <mergeCell ref="E94:E97"/>
+    <mergeCell ref="H182:H185"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="C34:C37"/>
+    <mergeCell ref="D10:D13"/>
+    <mergeCell ref="F10:F13"/>
+    <mergeCell ref="G14:G17"/>
+    <mergeCell ref="D18:D21"/>
+    <mergeCell ref="B178:B181"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="F66:F69"/>
+    <mergeCell ref="B74:B77"/>
+    <mergeCell ref="A42:A45"/>
+    <mergeCell ref="F38:F41"/>
+    <mergeCell ref="E162:E165"/>
+    <mergeCell ref="D130:D133"/>
+    <mergeCell ref="A134:A137"/>
+    <mergeCell ref="F130:F133"/>
+    <mergeCell ref="A126:A129"/>
+    <mergeCell ref="F106:F109"/>
+    <mergeCell ref="E142:E145"/>
+    <mergeCell ref="F118:F121"/>
+    <mergeCell ref="E158:E161"/>
+    <mergeCell ref="F178:F181"/>
+    <mergeCell ref="C178:C181"/>
+    <mergeCell ref="E178:E181"/>
+    <mergeCell ref="H162:H165"/>
+    <mergeCell ref="E138:E141"/>
+    <mergeCell ref="A118:A121"/>
+    <mergeCell ref="F114:F117"/>
+    <mergeCell ref="C118:C121"/>
+    <mergeCell ref="H114:H117"/>
+    <mergeCell ref="H70:H73"/>
+    <mergeCell ref="D66:D69"/>
+    <mergeCell ref="B186:B189"/>
+    <mergeCell ref="B142:B145"/>
+    <mergeCell ref="G138:G141"/>
+    <mergeCell ref="E174:E177"/>
+    <mergeCell ref="D142:D145"/>
+    <mergeCell ref="A186:A189"/>
+    <mergeCell ref="C186:C189"/>
+    <mergeCell ref="H82:H85"/>
+    <mergeCell ref="H118:H121"/>
+    <mergeCell ref="A182:A185"/>
+    <mergeCell ref="G182:G185"/>
+    <mergeCell ref="D178:D181"/>
+    <mergeCell ref="B114:B117"/>
+    <mergeCell ref="D114:D117"/>
+    <mergeCell ref="F170:F173"/>
+    <mergeCell ref="H170:H173"/>
+    <mergeCell ref="F190:F193"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="H190:H193"/>
+    <mergeCell ref="D30:D33"/>
+    <mergeCell ref="A106:A109"/>
+    <mergeCell ref="H14:H17"/>
+    <mergeCell ref="B54:B57"/>
+    <mergeCell ref="G42:G45"/>
+    <mergeCell ref="B94:B97"/>
+    <mergeCell ref="C126:C129"/>
+    <mergeCell ref="H122:H125"/>
+    <mergeCell ref="E126:E129"/>
+    <mergeCell ref="B102:B105"/>
+    <mergeCell ref="E190:E193"/>
+    <mergeCell ref="D158:D161"/>
+    <mergeCell ref="G190:G193"/>
+    <mergeCell ref="H74:H77"/>
+    <mergeCell ref="A50:A53"/>
+    <mergeCell ref="C50:C53"/>
+    <mergeCell ref="H46:H49"/>
+    <mergeCell ref="H26:H29"/>
+    <mergeCell ref="C42:C45"/>
+    <mergeCell ref="H38:H41"/>
+    <mergeCell ref="F74:F77"/>
+    <mergeCell ref="H198:H201"/>
+    <mergeCell ref="D42:D45"/>
+    <mergeCell ref="G90:G93"/>
+    <mergeCell ref="D94:D97"/>
+    <mergeCell ref="A114:A117"/>
+    <mergeCell ref="A170:A173"/>
+    <mergeCell ref="A70:A73"/>
+    <mergeCell ref="C170:C173"/>
+    <mergeCell ref="F158:F161"/>
+    <mergeCell ref="H54:H57"/>
+    <mergeCell ref="A166:A169"/>
+    <mergeCell ref="A178:A181"/>
+    <mergeCell ref="H154:H157"/>
+    <mergeCell ref="B194:B197"/>
+    <mergeCell ref="A174:A177"/>
+    <mergeCell ref="A194:A197"/>
+    <mergeCell ref="D118:D121"/>
+    <mergeCell ref="B126:B129"/>
+    <mergeCell ref="D182:D185"/>
+    <mergeCell ref="F182:F185"/>
+    <mergeCell ref="C74:C77"/>
+    <mergeCell ref="A110:A113"/>
+    <mergeCell ref="F162:F165"/>
+    <mergeCell ref="C166:C169"/>
+    <mergeCell ref="C158:C161"/>
+    <mergeCell ref="B50:B53"/>
+    <mergeCell ref="E38:E41"/>
+    <mergeCell ref="G38:G41"/>
+    <mergeCell ref="G98:G101"/>
+    <mergeCell ref="D174:D177"/>
+    <mergeCell ref="F174:F177"/>
+    <mergeCell ref="D166:D169"/>
+    <mergeCell ref="B118:B121"/>
+    <mergeCell ref="E130:E133"/>
+    <mergeCell ref="B134:B137"/>
+    <mergeCell ref="G130:G133"/>
+    <mergeCell ref="G114:G117"/>
+    <mergeCell ref="G62:G65"/>
+    <mergeCell ref="E42:E45"/>
+    <mergeCell ref="B106:B109"/>
+    <mergeCell ref="B170:B173"/>
+    <mergeCell ref="D170:D173"/>
+    <mergeCell ref="F138:F141"/>
+    <mergeCell ref="C142:C145"/>
+    <mergeCell ref="G166:G169"/>
+    <mergeCell ref="D150:D153"/>
+    <mergeCell ref="C154:C157"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="C2:C5"/>
+    <mergeCell ref="E2:E5"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="D98:D101"/>
+    <mergeCell ref="C66:C69"/>
+    <mergeCell ref="H62:H65"/>
+    <mergeCell ref="F98:F101"/>
+    <mergeCell ref="A102:A105"/>
+    <mergeCell ref="E66:E69"/>
+    <mergeCell ref="C102:C105"/>
+    <mergeCell ref="D50:D53"/>
+    <mergeCell ref="G86:G89"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="D2:D5"/>
+    <mergeCell ref="F18:F21"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="F22:F25"/>
+    <mergeCell ref="H22:H25"/>
+    <mergeCell ref="E54:E57"/>
+    <mergeCell ref="G54:G57"/>
+    <mergeCell ref="H86:H89"/>
+    <mergeCell ref="D38:D41"/>
+    <mergeCell ref="A58:A61"/>
+    <mergeCell ref="C194:C197"/>
+    <mergeCell ref="G110:G113"/>
+    <mergeCell ref="H150:H153"/>
+    <mergeCell ref="C18:C21"/>
+    <mergeCell ref="E18:E21"/>
+    <mergeCell ref="B150:B153"/>
+    <mergeCell ref="B190:B193"/>
+    <mergeCell ref="C26:C29"/>
+    <mergeCell ref="D190:D193"/>
+    <mergeCell ref="E82:E85"/>
+    <mergeCell ref="G82:G85"/>
+    <mergeCell ref="H102:H105"/>
+    <mergeCell ref="G146:G149"/>
+    <mergeCell ref="D122:D125"/>
+    <mergeCell ref="C90:C93"/>
+    <mergeCell ref="F122:F125"/>
+    <mergeCell ref="C182:C185"/>
+    <mergeCell ref="H178:H181"/>
+    <mergeCell ref="E182:E185"/>
+    <mergeCell ref="F186:F189"/>
+    <mergeCell ref="H42:H45"/>
+    <mergeCell ref="G194:G197"/>
+    <mergeCell ref="H50:H53"/>
+    <mergeCell ref="H142:H145"/>
+    <mergeCell ref="A190:A193"/>
+    <mergeCell ref="C190:C193"/>
+    <mergeCell ref="D74:D77"/>
+    <mergeCell ref="B138:B141"/>
+    <mergeCell ref="D138:D141"/>
+    <mergeCell ref="A142:A145"/>
+    <mergeCell ref="C14:C17"/>
+    <mergeCell ref="E14:E17"/>
+    <mergeCell ref="G70:G73"/>
+    <mergeCell ref="E30:E33"/>
+    <mergeCell ref="A46:A49"/>
+    <mergeCell ref="C46:C49"/>
+    <mergeCell ref="D14:D17"/>
+    <mergeCell ref="F14:F17"/>
+    <mergeCell ref="D86:D89"/>
+    <mergeCell ref="F86:F89"/>
+    <mergeCell ref="F142:F145"/>
+    <mergeCell ref="G18:G21"/>
+    <mergeCell ref="E34:E37"/>
+    <mergeCell ref="B182:B185"/>
+    <mergeCell ref="G34:G37"/>
+    <mergeCell ref="D162:D165"/>
+    <mergeCell ref="C130:C133"/>
+    <mergeCell ref="G30:G33"/>
     <mergeCell ref="D198:D201"/>
     <mergeCell ref="F198:F201"/>
     <mergeCell ref="A74:A77"/>
@@ -4222,331 +4480,78 @@
     <mergeCell ref="G170:G173"/>
     <mergeCell ref="D90:D93"/>
     <mergeCell ref="E194:E197"/>
-    <mergeCell ref="A190:A193"/>
-    <mergeCell ref="C190:C193"/>
-    <mergeCell ref="D74:D77"/>
-    <mergeCell ref="B138:B141"/>
-    <mergeCell ref="D138:D141"/>
-    <mergeCell ref="A142:A145"/>
-    <mergeCell ref="C14:C17"/>
-    <mergeCell ref="E14:E17"/>
-    <mergeCell ref="G70:G73"/>
-    <mergeCell ref="E30:E33"/>
-    <mergeCell ref="A46:A49"/>
-    <mergeCell ref="C46:C49"/>
-    <mergeCell ref="D14:D17"/>
-    <mergeCell ref="F14:F17"/>
-    <mergeCell ref="D86:D89"/>
-    <mergeCell ref="F86:F89"/>
-    <mergeCell ref="F142:F145"/>
-    <mergeCell ref="G18:G21"/>
-    <mergeCell ref="E34:E37"/>
-    <mergeCell ref="B182:B185"/>
-    <mergeCell ref="G34:G37"/>
-    <mergeCell ref="D162:D165"/>
-    <mergeCell ref="C130:C133"/>
-    <mergeCell ref="G30:G33"/>
-    <mergeCell ref="C194:C197"/>
-    <mergeCell ref="G110:G113"/>
-    <mergeCell ref="H150:H153"/>
-    <mergeCell ref="C18:C21"/>
-    <mergeCell ref="E18:E21"/>
-    <mergeCell ref="B150:B153"/>
-    <mergeCell ref="B190:B193"/>
-    <mergeCell ref="C26:C29"/>
-    <mergeCell ref="D190:D193"/>
-    <mergeCell ref="E82:E85"/>
-    <mergeCell ref="G82:G85"/>
-    <mergeCell ref="H102:H105"/>
-    <mergeCell ref="G146:G149"/>
-    <mergeCell ref="D122:D125"/>
-    <mergeCell ref="C90:C93"/>
-    <mergeCell ref="F122:F125"/>
-    <mergeCell ref="C182:C185"/>
-    <mergeCell ref="H178:H181"/>
-    <mergeCell ref="E182:E185"/>
-    <mergeCell ref="F186:F189"/>
-    <mergeCell ref="H42:H45"/>
-    <mergeCell ref="G194:G197"/>
-    <mergeCell ref="H50:H53"/>
-    <mergeCell ref="H142:H145"/>
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="C2:C5"/>
-    <mergeCell ref="E2:E5"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="D98:D101"/>
-    <mergeCell ref="C66:C69"/>
-    <mergeCell ref="H62:H65"/>
-    <mergeCell ref="F98:F101"/>
-    <mergeCell ref="A102:A105"/>
-    <mergeCell ref="E66:E69"/>
-    <mergeCell ref="C102:C105"/>
-    <mergeCell ref="D50:D53"/>
-    <mergeCell ref="G86:G89"/>
-    <mergeCell ref="B2:B5"/>
-    <mergeCell ref="D2:D5"/>
-    <mergeCell ref="F18:F21"/>
-    <mergeCell ref="B58:B61"/>
-    <mergeCell ref="F22:F25"/>
-    <mergeCell ref="H22:H25"/>
-    <mergeCell ref="E54:E57"/>
-    <mergeCell ref="G54:G57"/>
-    <mergeCell ref="H86:H89"/>
-    <mergeCell ref="D38:D41"/>
-    <mergeCell ref="A58:A61"/>
-    <mergeCell ref="D6:D9"/>
+    <mergeCell ref="H186:H189"/>
+    <mergeCell ref="D26:D29"/>
+    <mergeCell ref="D82:D85"/>
+    <mergeCell ref="F82:F85"/>
+    <mergeCell ref="H30:H33"/>
+    <mergeCell ref="B90:B93"/>
+    <mergeCell ref="A94:A97"/>
+    <mergeCell ref="F146:F149"/>
+    <mergeCell ref="H146:H149"/>
+    <mergeCell ref="G126:G129"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="H58:H61"/>
+    <mergeCell ref="E122:E125"/>
+    <mergeCell ref="E78:E81"/>
+    <mergeCell ref="G122:G125"/>
+    <mergeCell ref="G78:G81"/>
+    <mergeCell ref="C134:C137"/>
+    <mergeCell ref="E186:E189"/>
     <mergeCell ref="G178:G181"/>
-    <mergeCell ref="F6:F9"/>
     <mergeCell ref="B62:B65"/>
     <mergeCell ref="E98:E101"/>
     <mergeCell ref="G162:G165"/>
     <mergeCell ref="C150:C153"/>
+    <mergeCell ref="E134:E137"/>
+    <mergeCell ref="A158:A161"/>
+    <mergeCell ref="G174:G177"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="E46:E49"/>
+    <mergeCell ref="D106:D109"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="E86:E89"/>
+    <mergeCell ref="B162:B165"/>
+    <mergeCell ref="G150:G153"/>
+    <mergeCell ref="G94:G97"/>
+    <mergeCell ref="G158:G161"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="D22:D25"/>
+    <mergeCell ref="F78:F81"/>
+    <mergeCell ref="B86:B89"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="G58:G61"/>
+    <mergeCell ref="A150:A153"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="C22:C25"/>
+    <mergeCell ref="D6:D9"/>
+    <mergeCell ref="F6:F9"/>
     <mergeCell ref="E22:E25"/>
     <mergeCell ref="G22:G25"/>
-    <mergeCell ref="E134:E137"/>
+    <mergeCell ref="C6:C9"/>
+    <mergeCell ref="C62:C65"/>
+    <mergeCell ref="E62:E65"/>
+    <mergeCell ref="H6:H9"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="H98:H101"/>
+    <mergeCell ref="A66:A69"/>
+    <mergeCell ref="B98:B101"/>
+    <mergeCell ref="D154:D157"/>
+    <mergeCell ref="F154:F157"/>
+    <mergeCell ref="H126:H129"/>
+    <mergeCell ref="H78:H81"/>
+    <mergeCell ref="H10:H13"/>
     <mergeCell ref="F54:F57"/>
-    <mergeCell ref="C158:C161"/>
-    <mergeCell ref="B50:B53"/>
-    <mergeCell ref="E38:E41"/>
-    <mergeCell ref="G38:G41"/>
-    <mergeCell ref="G98:G101"/>
-    <mergeCell ref="D174:D177"/>
-    <mergeCell ref="F174:F177"/>
-    <mergeCell ref="D166:D169"/>
-    <mergeCell ref="B118:B121"/>
-    <mergeCell ref="E130:E133"/>
-    <mergeCell ref="B134:B137"/>
-    <mergeCell ref="G130:G133"/>
-    <mergeCell ref="G114:G117"/>
-    <mergeCell ref="H198:H201"/>
-    <mergeCell ref="D42:D45"/>
-    <mergeCell ref="G90:G93"/>
-    <mergeCell ref="D94:D97"/>
-    <mergeCell ref="A114:A117"/>
-    <mergeCell ref="A170:A173"/>
-    <mergeCell ref="A70:A73"/>
-    <mergeCell ref="C170:C173"/>
-    <mergeCell ref="F158:F161"/>
-    <mergeCell ref="H54:H57"/>
-    <mergeCell ref="A166:A169"/>
-    <mergeCell ref="A178:A181"/>
-    <mergeCell ref="H154:H157"/>
-    <mergeCell ref="B194:B197"/>
-    <mergeCell ref="A174:A177"/>
-    <mergeCell ref="A194:A197"/>
-    <mergeCell ref="D118:D121"/>
-    <mergeCell ref="B126:B129"/>
-    <mergeCell ref="D182:D185"/>
-    <mergeCell ref="F182:F185"/>
-    <mergeCell ref="C74:C77"/>
-    <mergeCell ref="A110:A113"/>
-    <mergeCell ref="F162:F165"/>
-    <mergeCell ref="C166:C169"/>
     <mergeCell ref="E6:E9"/>
     <mergeCell ref="G6:G9"/>
-    <mergeCell ref="G62:G65"/>
     <mergeCell ref="A154:A157"/>
-    <mergeCell ref="F190:F193"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="H190:H193"/>
-    <mergeCell ref="D30:D33"/>
-    <mergeCell ref="A106:A109"/>
-    <mergeCell ref="H14:H17"/>
-    <mergeCell ref="B54:B57"/>
-    <mergeCell ref="G42:G45"/>
-    <mergeCell ref="B94:B97"/>
-    <mergeCell ref="C126:C129"/>
-    <mergeCell ref="H122:H125"/>
-    <mergeCell ref="E126:E129"/>
-    <mergeCell ref="B102:B105"/>
-    <mergeCell ref="E190:E193"/>
-    <mergeCell ref="D158:D161"/>
-    <mergeCell ref="G190:G193"/>
-    <mergeCell ref="H74:H77"/>
-    <mergeCell ref="A50:A53"/>
-    <mergeCell ref="C50:C53"/>
-    <mergeCell ref="H46:H49"/>
-    <mergeCell ref="H26:H29"/>
-    <mergeCell ref="C42:C45"/>
-    <mergeCell ref="H38:H41"/>
-    <mergeCell ref="F74:F77"/>
     <mergeCell ref="A78:A81"/>
-    <mergeCell ref="E42:E45"/>
     <mergeCell ref="H130:H133"/>
-    <mergeCell ref="B106:B109"/>
-    <mergeCell ref="B170:B173"/>
-    <mergeCell ref="D170:D173"/>
     <mergeCell ref="A86:A89"/>
-    <mergeCell ref="F138:F141"/>
-    <mergeCell ref="C142:C145"/>
     <mergeCell ref="H138:H141"/>
     <mergeCell ref="B34:B37"/>
     <mergeCell ref="H34:H37"/>
-    <mergeCell ref="H162:H165"/>
-    <mergeCell ref="E138:E141"/>
-    <mergeCell ref="A118:A121"/>
-    <mergeCell ref="F114:F117"/>
-    <mergeCell ref="C118:C121"/>
-    <mergeCell ref="H114:H117"/>
-    <mergeCell ref="H70:H73"/>
-    <mergeCell ref="D66:D69"/>
-    <mergeCell ref="B186:B189"/>
-    <mergeCell ref="B142:B145"/>
-    <mergeCell ref="G138:G141"/>
-    <mergeCell ref="E174:E177"/>
-    <mergeCell ref="D142:D145"/>
     <mergeCell ref="E26:E29"/>
-    <mergeCell ref="A34:A37"/>
-    <mergeCell ref="C34:C37"/>
-    <mergeCell ref="D10:D13"/>
-    <mergeCell ref="F10:F13"/>
-    <mergeCell ref="G14:G17"/>
-    <mergeCell ref="D18:D21"/>
-    <mergeCell ref="B178:B181"/>
-    <mergeCell ref="B10:B13"/>
-    <mergeCell ref="F66:F69"/>
-    <mergeCell ref="B74:B77"/>
-    <mergeCell ref="A42:A45"/>
-    <mergeCell ref="F38:F41"/>
-    <mergeCell ref="E162:E165"/>
-    <mergeCell ref="D130:D133"/>
-    <mergeCell ref="A134:A137"/>
-    <mergeCell ref="F130:F133"/>
-    <mergeCell ref="A126:A129"/>
-    <mergeCell ref="F106:F109"/>
-    <mergeCell ref="D194:D197"/>
-    <mergeCell ref="F134:F137"/>
-    <mergeCell ref="A198:A201"/>
-    <mergeCell ref="F194:F197"/>
-    <mergeCell ref="C198:C201"/>
-    <mergeCell ref="H194:H197"/>
-    <mergeCell ref="C110:C113"/>
-    <mergeCell ref="H18:H21"/>
-    <mergeCell ref="B154:B157"/>
-    <mergeCell ref="C174:C177"/>
-    <mergeCell ref="G46:G49"/>
-    <mergeCell ref="H106:H109"/>
-    <mergeCell ref="A30:A33"/>
-    <mergeCell ref="C30:C33"/>
-    <mergeCell ref="A54:A57"/>
-    <mergeCell ref="C54:C57"/>
-    <mergeCell ref="A90:A93"/>
-    <mergeCell ref="A146:A149"/>
-    <mergeCell ref="C146:C149"/>
-    <mergeCell ref="D126:D129"/>
-    <mergeCell ref="C94:C97"/>
-    <mergeCell ref="F126:F129"/>
-    <mergeCell ref="E94:E97"/>
-    <mergeCell ref="H182:H185"/>
-    <mergeCell ref="A186:A189"/>
-    <mergeCell ref="C186:C189"/>
-    <mergeCell ref="E142:E145"/>
-    <mergeCell ref="H82:H85"/>
-    <mergeCell ref="F118:F121"/>
-    <mergeCell ref="H118:H121"/>
-    <mergeCell ref="G2:G5"/>
-    <mergeCell ref="A138:A141"/>
-    <mergeCell ref="C10:C13"/>
-    <mergeCell ref="E10:E13"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="B70:B73"/>
-    <mergeCell ref="G10:G13"/>
-    <mergeCell ref="G66:G69"/>
-    <mergeCell ref="D70:D73"/>
-    <mergeCell ref="F70:F73"/>
-    <mergeCell ref="D134:D137"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="E158:E161"/>
-    <mergeCell ref="F46:F49"/>
-    <mergeCell ref="E74:E77"/>
-    <mergeCell ref="B78:B81"/>
-    <mergeCell ref="F42:F45"/>
-    <mergeCell ref="G74:G77"/>
-    <mergeCell ref="B198:B201"/>
-    <mergeCell ref="A38:A41"/>
-    <mergeCell ref="A130:A133"/>
-    <mergeCell ref="B110:B113"/>
-    <mergeCell ref="D110:D113"/>
-    <mergeCell ref="E146:E149"/>
-    <mergeCell ref="F166:F169"/>
-    <mergeCell ref="C58:C61"/>
-    <mergeCell ref="E58:E61"/>
-    <mergeCell ref="D186:D189"/>
-    <mergeCell ref="B82:B85"/>
-    <mergeCell ref="F90:F93"/>
-    <mergeCell ref="E118:E121"/>
-    <mergeCell ref="B146:B149"/>
-    <mergeCell ref="D146:D149"/>
-    <mergeCell ref="E166:E169"/>
-    <mergeCell ref="F50:F53"/>
-    <mergeCell ref="C38:C41"/>
-    <mergeCell ref="D58:D61"/>
-    <mergeCell ref="A62:A65"/>
-    <mergeCell ref="F58:F61"/>
-    <mergeCell ref="A122:A125"/>
-    <mergeCell ref="C122:C125"/>
-    <mergeCell ref="C78:C81"/>
-    <mergeCell ref="A182:A185"/>
-    <mergeCell ref="F178:F181"/>
-    <mergeCell ref="B18:B21"/>
-    <mergeCell ref="F34:F37"/>
-    <mergeCell ref="F2:F5"/>
-    <mergeCell ref="H2:H5"/>
-    <mergeCell ref="H94:H97"/>
-    <mergeCell ref="C114:C117"/>
-    <mergeCell ref="C70:C73"/>
-    <mergeCell ref="E114:E117"/>
-    <mergeCell ref="E170:E173"/>
-    <mergeCell ref="F102:F105"/>
-    <mergeCell ref="E70:E73"/>
-    <mergeCell ref="H66:H69"/>
-    <mergeCell ref="C106:C109"/>
-    <mergeCell ref="C178:C181"/>
-    <mergeCell ref="E178:E181"/>
-    <mergeCell ref="D62:D65"/>
-    <mergeCell ref="F62:F65"/>
-    <mergeCell ref="F26:F29"/>
-    <mergeCell ref="H90:H93"/>
-    <mergeCell ref="G118:G121"/>
-    <mergeCell ref="G182:G185"/>
-    <mergeCell ref="A14:A17"/>
-    <mergeCell ref="H158:H161"/>
-    <mergeCell ref="E50:E53"/>
-    <mergeCell ref="C86:C89"/>
-    <mergeCell ref="G50:G53"/>
-    <mergeCell ref="D54:D57"/>
-    <mergeCell ref="B122:B125"/>
-    <mergeCell ref="E150:E153"/>
-    <mergeCell ref="D178:D181"/>
-    <mergeCell ref="D34:D37"/>
-    <mergeCell ref="G134:G137"/>
-    <mergeCell ref="H166:H169"/>
-    <mergeCell ref="E110:E113"/>
-    <mergeCell ref="D78:D81"/>
-    <mergeCell ref="B114:B117"/>
-    <mergeCell ref="D114:D117"/>
-    <mergeCell ref="F170:F173"/>
-    <mergeCell ref="H170:H173"/>
-    <mergeCell ref="G166:G169"/>
-    <mergeCell ref="D150:D153"/>
-    <mergeCell ref="A98:A101"/>
-    <mergeCell ref="F150:F153"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="F94:F97"/>
-    <mergeCell ref="G26:G29"/>
-    <mergeCell ref="C82:C85"/>
-    <mergeCell ref="D102:D105"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="B66:B69"/>
-    <mergeCell ref="C154:C157"/>
-    <mergeCell ref="C98:C101"/>
-    <mergeCell ref="E102:E105"/>
-    <mergeCell ref="G102:G105"/>
-    <mergeCell ref="A162:A165"/>
-    <mergeCell ref="F30:F33"/>
-    <mergeCell ref="C162:C165"/>
-    <mergeCell ref="B130:B133"/>
-    <mergeCell ref="D46:D49"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>